<commit_message>
fix: Updated debugg manual openpyxl.
</commit_message>
<xml_diff>
--- a/SmartBU/How_To_Debugg.xlsx
+++ b/SmartBU/How_To_Debugg.xlsx
@@ -1,12 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UShin\Testbench_gui_Charan\SmartBU\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14130"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="MXAj33uNO1zcz6WY6d6qq3mLHNVLbJybT5QnkKJAJAQ="/>
@@ -16,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>Project Setup Using Trace32</t>
   </si>
@@ -44,25 +52,26 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve">Download the </t>
     </r>
     <r>
       <rPr>
-        <rFont val="Calibri"/>
         <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
       </rPr>
       <t>Trace32 setup package and Python installer</t>
     </r>
     <r>
       <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve"> from the following Google Drive link:</t>
     </r>
@@ -79,562 +88,596 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve">2. Run </t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>setupt.bat</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>3. Follow the on-screen instructions to complete the installation.</t>
+  </si>
+  <si>
+    <t>4. Install Python</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">1. Run </t>
+    </r>
+    <r>
+      <rPr>
         <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
-      </rPr>
-      <t>setupt.bat</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>python-3.14.2-amd64.exe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
       </rPr>
       <t>.</t>
     </r>
   </si>
   <si>
-    <t>3. Follow the on-screen instructions to complete the installation.</t>
-  </si>
-  <si>
-    <t>4. Install Python</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">1. Run </t>
-    </r>
-    <r>
-      <rPr>
+    <t>2. During installation:</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">✅ Check </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>“Add Python to PATH”</t>
+    </r>
+  </si>
+  <si>
+    <t>3. Complete the installation.</t>
+  </si>
+  <si>
+    <t>5. Install Python Dependencies</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">Open </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Command Prompt (CMD)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> and run the following commands one by one:</t>
+    </r>
+  </si>
+  <si>
+    <t>pip install pyvisa</t>
+  </si>
+  <si>
+    <t>pip install pyvisa-py</t>
+  </si>
+  <si>
+    <t>pip install Lauterbach.trace32.rcl</t>
+  </si>
+  <si>
+    <t>Verify that all packages are installed without errors.</t>
+  </si>
+  <si>
+    <t>6. Download the Project</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">Download the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>SmartBU Project</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> from the following Google Drive link:</t>
+    </r>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/1gTF1ggrcZLFDnWPfuxJlCGeO36il9DKW</t>
+  </si>
+  <si>
+    <t>7. Change T32 Installation path in Project.</t>
+  </si>
+  <si>
+    <t>Change path according the T32 installion directory</t>
+  </si>
+  <si>
+    <t>1. Update Config.t32 : line number "4".</t>
+  </si>
+  <si>
+    <t>For eg:</t>
+  </si>
+  <si>
+    <t>SYS=C:\Users\Nverma\.conan2\p\tracee4f08930e322b\p</t>
+  </si>
+  <si>
+    <t>SYS=C:\T32</t>
+  </si>
+  <si>
+    <t>2. Update trace32.py : line number "134". Installation path</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trace32_path = f"{user_path_cleaned}\\.conan2\\p\\tracee4f08930e322b\\p\\bin\\windows64\\t32marm.exe" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">trace32_path = r"C:\T32\bin\windows64\t32marm.exe" </t>
+  </si>
+  <si>
+    <t>3. Update trace32.py : line number "296".</t>
+  </si>
+  <si>
+    <t>new_path = f"{user_path_cleaned}\\.conan2\\p\\tracee4f08930e322b\\p"</t>
+  </si>
+  <si>
+    <t>new_path = r"C:\T32"</t>
+  </si>
+  <si>
+    <t>8. Hardware Connection and Application Launch</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">1. Connect the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Trace32 hardware</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> to the PC and target board.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">2. Open the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Testbench_gui</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> project directory.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">3. Run </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>SmartBuApp.bat.</t>
+    </r>
+  </si>
+  <si>
+    <t>9. Configure the Application</t>
+  </si>
+  <si>
+    <t>After launching the application, perform the following steps:</t>
+  </si>
+  <si>
+    <t>1. Select ELF File</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">Click </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Browse</t>
+    </r>
+  </si>
+  <si>
+    <t>Select the appropriate ELF file path (For example .. \Testbench_gui\SmartBU)</t>
+  </si>
+  <si>
+    <t>2. Select SmartBU Directory</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">Choose the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>SmartBU folder</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> from the project directory</t>
+    </r>
+  </si>
+  <si>
+    <t>3. Select Handle Variant</t>
+  </si>
+  <si>
+    <t>Select the variant according to your connected hardware</t>
+  </si>
+  <si>
+    <t>10. Connect and Start Execution</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">1. Click </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">“Connect Trace32” </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>and</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>wait for to status to change to "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>stopped at the breakpoint</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>"</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">2. Click </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>“Start Code”</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">3. Verify that the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>status changes to “Running”</t>
+    </r>
+  </si>
+  <si>
+    <t>✅ Successful connection confirms that Trace32 and the application are working correctly.</t>
+  </si>
+  <si>
+    <t>11. Disconnect and Stop execution</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">1. Before clossing Gui Click </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">"Disconnect Trace32" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>and wait for stautus to change to "none"</t>
+    </r>
+  </si>
+  <si>
+    <t>2. Close with X button on GUI</t>
+  </si>
+  <si>
+    <t>12. Troubleshooting</t>
+  </si>
+  <si>
+    <t>Ensure Trace32 drivers are correctly installed</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Confirm Python is accessible from CMD (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
-      </rPr>
-      <t>python-3.14.2-amd64.exe</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <t>2. During installation:</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">✅ Check </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>“Add Python to PATH”</t>
-    </r>
-  </si>
-  <si>
-    <t>3. Complete the installation.</t>
-  </si>
-  <si>
-    <t>5. Install Python Dependencies</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">Open </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>Command Prompt (CMD)</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> and run the following commands one by one:</t>
-    </r>
-  </si>
-  <si>
-    <t>pip install pyvisa</t>
-  </si>
-  <si>
-    <t>pip install pyvisa-py</t>
-  </si>
-  <si>
-    <t>pip install Lauterbach.trace32.rcl</t>
-  </si>
-  <si>
-    <t>Verify that all packages are installed without errors.</t>
-  </si>
-  <si>
-    <t>6. Download the Project</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">Download the </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>SmartBU Project</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> from the following Google Drive link:</t>
-    </r>
-  </si>
-  <si>
-    <t>https://drive.google.com/drive/folders/1gTF1ggrcZLFDnWPfuxJlCGeO36il9DKW</t>
-  </si>
-  <si>
-    <t>7. Change T32 Installation path in Project.</t>
-  </si>
-  <si>
-    <t>Change path according the T32 installion directory</t>
-  </si>
-  <si>
-    <t>1. Update Config.t32 : line number "4".</t>
-  </si>
-  <si>
-    <t>For eg:</t>
-  </si>
-  <si>
-    <t>SYS=C:\Users\Nverma\.conan2\p\tracee4f08930e322b\p</t>
-  </si>
-  <si>
-    <t>SYS=C:\T32</t>
-  </si>
-  <si>
-    <t>2. Update trace32.py : line number "134". Installation path</t>
-  </si>
-  <si>
-    <t xml:space="preserve">trace32_path = f"{user_path_cleaned}\\.conan2\\p\\tracee4f08930e322b\\p\\bin\\windows64\\t32marm.exe" </t>
-  </si>
-  <si>
-    <t xml:space="preserve">trace32_path = r"C:\T32\bin\windows64\t32marm.exe" </t>
-  </si>
-  <si>
-    <t>3. Update trace32.py : line number "296".</t>
-  </si>
-  <si>
-    <t>new_path = f"{user_path_cleaned}\\.conan2\\p\\tracee4f08930e322b\\p"</t>
-  </si>
-  <si>
-    <t>new_path = r"C:\T32"</t>
-  </si>
-  <si>
-    <t>8. Hardware Connection and Application Launch</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">1. Connect the </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>Trace32 hardware</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> to the PC and target board.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">2. Open the </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>Testbench_gui</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> project directory.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">3. Run </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>SmartBuApp.bat.</t>
-    </r>
-  </si>
-  <si>
-    <t>9. Configure the Application</t>
-  </si>
-  <si>
-    <t>After launching the application, perform the following steps:</t>
-  </si>
-  <si>
-    <t>1. Select ELF File</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">Click </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>Browse</t>
-    </r>
-  </si>
-  <si>
-    <t>Select the appropriate ELF file path (For example .. \Testbench_gui\SmartBU)</t>
-  </si>
-  <si>
-    <t>2. Select SmartBU Directory</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">Choose the </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>SmartBU folder</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> from the project directory</t>
-    </r>
-  </si>
-  <si>
-    <t>3. Select Handle Variant</t>
-  </si>
-  <si>
-    <t>Select the variant according to your connected hardware</t>
-  </si>
-  <si>
-    <t>10. Connect and Start Execution</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">1. Click </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">“Connect Trace32” </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>and</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>wait for to status to change to "</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color rgb="FFFF0000"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>stopped at the breakpoint</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>"</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">2. Click </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>“Start Code”</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">3. Verify that the </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>status changes to “Running”</t>
-    </r>
-  </si>
-  <si>
-    <t>✅ Successful connection confirms that Trace32 and the application are working correctly.</t>
-  </si>
-  <si>
-    <t>11. Disconnect and Stop execution</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">1. Before clossing Gui Click </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">"Disconnect Trace32" </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>and wait for stautus to change to "none"</t>
-    </r>
-  </si>
-  <si>
-    <t>2. Close with X button on GUI</t>
-  </si>
-  <si>
-    <t>12. Troubleshooting</t>
-  </si>
-  <si>
-    <t>Ensure Trace32 drivers are correctly installed</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>Confirm Python is accessible from CMD (</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial Unicode MS"/>
-        <color theme="1"/>
-        <sz val="10.0"/>
       </rPr>
       <t>python --version</t>
     </r>
     <r>
       <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
       </rPr>
       <t>)</t>
     </r>
   </si>
   <si>
     <t>Verify correct ELF and SmartBU paths</t>
+  </si>
+  <si>
+    <t>pip install openpyxl</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="13">
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="36"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="36.0"/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11.0"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arimo"/>
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF00B0F0"/>
+      <name val="Arimo"/>
     </font>
   </fonts>
   <fills count="2">
@@ -642,62 +685,78 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+  <cellXfs count="12">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="標準 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>12</xdr:col>
       <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>159</xdr:row>
+      <xdr:row>160</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1743075" cy="723900"/>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="3" name="Shape 3"/>
         <xdr:cNvSpPr/>
@@ -709,30 +768,30 @@
         </a:xfrm>
         <a:prstGeom prst="rightArrow">
           <a:avLst>
-            <a:gd fmla="val 50000" name="adj1"/>
-            <a:gd fmla="val 50000" name="adj2"/>
+            <a:gd name="adj1" fmla="val 50000"/>
+            <a:gd name="adj2" fmla="val 50000"/>
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
           <a:schemeClr val="accent1"/>
         </a:solidFill>
-        <a:ln cap="flat" cmpd="sng" w="12700">
+        <a:ln w="12700" cap="flat" cmpd="sng">
           <a:solidFill>
             <a:srgbClr val="42719B"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
-          <a:headEnd len="sm" w="sm" type="none"/>
-          <a:tailEnd len="sm" w="sm" type="none"/>
+          <a:headEnd type="none" w="sm" len="sm"/>
+          <a:tailEnd type="none" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
       <xdr:txBody>
-        <a:bodyPr anchorCtr="0" anchor="t" bIns="45700" lIns="91425" spcFirstLastPara="1" rIns="91425" wrap="square" tIns="45700">
+        <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="91425" tIns="45700" rIns="91425" bIns="45700" anchor="t" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr indent="0" lvl="0" marL="0" rtl="0" algn="l">
+          <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
             <a:spcBef>
               <a:spcPts val="0"/>
             </a:spcBef>
@@ -741,9 +800,6 @@
             </a:spcAft>
             <a:buNone/>
           </a:pPr>
-          <a:r>
-            <a:t/>
-          </a:r>
           <a:endParaRPr sz="1100"/>
         </a:p>
       </xdr:txBody>
@@ -754,13 +810,13 @@
     <xdr:from>
       <xdr:col>12</xdr:col>
       <xdr:colOff>323850</xdr:colOff>
-      <xdr:row>183</xdr:row>
+      <xdr:row>184</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1743075" cy="723900"/>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Shape 3"/>
+        <xdr:cNvPr id="2" name="Shape 3"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -770,30 +826,30 @@
         </a:xfrm>
         <a:prstGeom prst="rightArrow">
           <a:avLst>
-            <a:gd fmla="val 50000" name="adj1"/>
-            <a:gd fmla="val 50000" name="adj2"/>
+            <a:gd name="adj1" fmla="val 50000"/>
+            <a:gd name="adj2" fmla="val 50000"/>
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
           <a:schemeClr val="accent1"/>
         </a:solidFill>
-        <a:ln cap="flat" cmpd="sng" w="12700">
+        <a:ln w="12700" cap="flat" cmpd="sng">
           <a:solidFill>
             <a:srgbClr val="42719B"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
-          <a:headEnd len="sm" w="sm" type="none"/>
-          <a:tailEnd len="sm" w="sm" type="none"/>
+          <a:headEnd type="none" w="sm" len="sm"/>
+          <a:tailEnd type="none" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
       <xdr:txBody>
-        <a:bodyPr anchorCtr="0" anchor="t" bIns="45700" lIns="91425" spcFirstLastPara="1" rIns="91425" wrap="square" tIns="45700">
+        <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="91425" tIns="45700" rIns="91425" bIns="45700" anchor="t" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr indent="0" lvl="0" marL="0" rtl="0" algn="l">
+          <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
             <a:spcBef>
               <a:spcPts val="0"/>
             </a:spcBef>
@@ -802,9 +858,6 @@
             </a:spcAft>
             <a:buNone/>
           </a:pPr>
-          <a:r>
-            <a:t/>
-          </a:r>
           <a:endParaRPr sz="1100"/>
         </a:p>
       </xdr:txBody>
@@ -815,13 +868,13 @@
     <xdr:from>
       <xdr:col>12</xdr:col>
       <xdr:colOff>390525</xdr:colOff>
-      <xdr:row>209</xdr:row>
+      <xdr:row>210</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1743075" cy="723900"/>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Shape 3"/>
+        <xdr:cNvPr id="4" name="Shape 3"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -831,30 +884,30 @@
         </a:xfrm>
         <a:prstGeom prst="rightArrow">
           <a:avLst>
-            <a:gd fmla="val 50000" name="adj1"/>
-            <a:gd fmla="val 50000" name="adj2"/>
+            <a:gd name="adj1" fmla="val 50000"/>
+            <a:gd name="adj2" fmla="val 50000"/>
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
           <a:schemeClr val="accent1"/>
         </a:solidFill>
-        <a:ln cap="flat" cmpd="sng" w="12700">
+        <a:ln w="12700" cap="flat" cmpd="sng">
           <a:solidFill>
             <a:srgbClr val="42719B"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
-          <a:headEnd len="sm" w="sm" type="none"/>
-          <a:tailEnd len="sm" w="sm" type="none"/>
+          <a:headEnd type="none" w="sm" len="sm"/>
+          <a:tailEnd type="none" w="sm" len="sm"/>
         </a:ln>
       </xdr:spPr>
       <xdr:txBody>
-        <a:bodyPr anchorCtr="0" anchor="t" bIns="45700" lIns="91425" spcFirstLastPara="1" rIns="91425" wrap="square" tIns="45700">
+        <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="91425" tIns="45700" rIns="91425" bIns="45700" anchor="t" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr indent="0" lvl="0" marL="0" rtl="0" algn="l">
+          <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
             <a:spcBef>
               <a:spcPts val="0"/>
             </a:spcBef>
@@ -863,9 +916,6 @@
             </a:spcAft>
             <a:buNone/>
           </a:pPr>
-          <a:r>
-            <a:t/>
-          </a:r>
           <a:endParaRPr sz="1100"/>
         </a:p>
       </xdr:txBody>
@@ -882,11 +932,11 @@
     <xdr:ext cx="6162675" cy="2924175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png"/>
+        <xdr:cNvPr id="5" name="image5.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -910,11 +960,11 @@
     <xdr:ext cx="6343650" cy="2971800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png"/>
+        <xdr:cNvPr id="6" name="image2.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -932,17 +982,17 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>98</xdr:row>
       <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6343650" cy="3409950"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image6.png"/>
+        <xdr:cNvPr id="7" name="image6.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -966,11 +1016,11 @@
     <xdr:ext cx="6334125" cy="3305175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image12.png"/>
+        <xdr:cNvPr id="8" name="image12.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -988,17 +1038,17 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>230</xdr:row>
+      <xdr:row>231</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6343650" cy="3209925"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image11.png"/>
+        <xdr:cNvPr id="9" name="image11.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1016,17 +1066,17 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>258</xdr:row>
+      <xdr:row>259</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6296025" cy="4171950"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png"/>
+        <xdr:cNvPr id="10" name="image3.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1044,17 +1094,17 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>286</xdr:row>
+      <xdr:row>287</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6296025" cy="4619625"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image15.png"/>
+        <xdr:cNvPr id="11" name="image15.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1072,17 +1122,17 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>124</xdr:row>
+      <xdr:row>125</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6457950" cy="3333750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image7.png"/>
+        <xdr:cNvPr id="12" name="image7.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1100,17 +1150,17 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>175</xdr:row>
+      <xdr:row>176</xdr:row>
       <xdr:rowOff>142875</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6400800" cy="3829050"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image9.png"/>
+        <xdr:cNvPr id="13" name="image9.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1128,17 +1178,17 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>151</xdr:row>
+      <xdr:row>152</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6362700" cy="3810000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image10.png"/>
+        <xdr:cNvPr id="14" name="image10.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1156,17 +1206,17 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>201</xdr:row>
+      <xdr:row>202</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6467475" cy="3829050"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image17.png"/>
+        <xdr:cNvPr id="15" name="image17.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1184,17 +1234,17 @@
     <xdr:from>
       <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>151</xdr:row>
+      <xdr:row>152</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6267450" cy="3714750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png"/>
+        <xdr:cNvPr id="16" name="image1.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1212,17 +1262,17 @@
     <xdr:from>
       <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>176</xdr:row>
+      <xdr:row>177</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6238875" cy="3676650"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image14.png"/>
+        <xdr:cNvPr id="17" name="image14.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1240,17 +1290,17 @@
     <xdr:from>
       <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>201</xdr:row>
+      <xdr:row>202</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6296025" cy="3914775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image16.png"/>
+        <xdr:cNvPr id="18" name="image16.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1268,17 +1318,17 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>571500</xdr:colOff>
-      <xdr:row>314</xdr:row>
+      <xdr:row>315</xdr:row>
       <xdr:rowOff>190500</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6296025" cy="4191000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.png" title="Image"/>
+        <xdr:cNvPr id="19" name="image4.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1296,17 +1346,17 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>581025</xdr:colOff>
-      <xdr:row>346</xdr:row>
+      <xdr:row>347</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6591300" cy="4429125"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image13.png" title="Image"/>
+        <xdr:cNvPr id="20" name="image13.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1324,17 +1374,17 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>377</xdr:row>
+      <xdr:row>378</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6362700" cy="4848225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image8.png" title="Image"/>
+        <xdr:cNvPr id="21" name="image8.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1352,7 +1402,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1542,267 +1592,271 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B1:Q1004"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="27" width="8.71"/>
+    <col min="1" max="27" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1"/>
-    <row r="2" ht="14.25" customHeight="1">
+    <row r="1" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="2" spans="2:2" ht="14.25" customHeight="1">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1">
+    <row r="3" spans="2:2" ht="14.25" customHeight="1">
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" ht="14.25" customHeight="1"/>
-    <row r="5" ht="14.25" customHeight="1"/>
-    <row r="6" ht="14.25" customHeight="1"/>
-    <row r="7" ht="14.25" customHeight="1">
+    <row r="4" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="5" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="6" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="7" spans="2:2" ht="14.25" customHeight="1">
       <c r="B7" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" ht="14.25" customHeight="1"/>
-    <row r="9" ht="14.25" customHeight="1">
+    <row r="8" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="9" spans="2:2" ht="14.25" customHeight="1">
       <c r="B9" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" ht="14.25" customHeight="1">
+    <row r="10" spans="2:2" ht="14.25" customHeight="1">
       <c r="B10" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" ht="14.25" customHeight="1">
+    <row r="11" spans="2:2" ht="14.25" customHeight="1">
       <c r="B11" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" ht="14.25" customHeight="1">
+    <row r="12" spans="2:2" ht="14.25" customHeight="1">
       <c r="B12" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" ht="14.25" customHeight="1">
+    <row r="13" spans="2:2" ht="14.25" customHeight="1">
       <c r="B13" s="4"/>
     </row>
-    <row r="14" ht="14.25" customHeight="1"/>
-    <row r="15" ht="14.25" customHeight="1">
+    <row r="14" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="15" spans="2:2" ht="14.25" customHeight="1">
       <c r="B15" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" ht="14.25" customHeight="1"/>
-    <row r="17" ht="14.25" customHeight="1">
+    <row r="16" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="17" spans="2:2" ht="14.25" customHeight="1">
       <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1">
+    <row r="18" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="19" spans="2:2" ht="14.25" customHeight="1">
       <c r="B19" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
-    <row r="33" ht="14.25" customHeight="1"/>
-    <row r="34" ht="14.25" customHeight="1"/>
-    <row r="35" ht="14.25" customHeight="1"/>
-    <row r="36" ht="14.25" customHeight="1"/>
-    <row r="37" ht="14.25" customHeight="1"/>
-    <row r="38" ht="14.25" customHeight="1">
+    <row r="20" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="21" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="22" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="23" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="24" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="25" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="26" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="27" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="28" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="29" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="30" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="31" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="32" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="33" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="34" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="35" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="36" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="37" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="38" spans="2:2" ht="14.25" customHeight="1">
       <c r="B38" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="39" ht="14.25" customHeight="1">
+    <row r="39" spans="2:2" ht="14.25" customHeight="1">
       <c r="B39" s="4"/>
     </row>
-    <row r="40" ht="14.25" customHeight="1">
+    <row r="40" spans="2:2" ht="14.25" customHeight="1">
       <c r="B40" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="41" ht="14.25" customHeight="1">
+    <row r="41" spans="2:2" ht="14.25" customHeight="1">
       <c r="B41" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="42" ht="14.25" customHeight="1">
+    <row r="42" spans="2:2" ht="14.25" customHeight="1">
       <c r="B42" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="43" ht="14.25" customHeight="1"/>
-    <row r="44" ht="14.25" customHeight="1"/>
-    <row r="45" ht="14.25" customHeight="1"/>
-    <row r="46" ht="14.25" customHeight="1"/>
-    <row r="47" ht="14.25" customHeight="1"/>
-    <row r="48" ht="14.25" customHeight="1"/>
-    <row r="49" ht="14.25" customHeight="1"/>
-    <row r="50" ht="14.25" customHeight="1"/>
-    <row r="51" ht="14.25" customHeight="1"/>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
-    <row r="62" ht="14.25" customHeight="1">
+    <row r="43" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="44" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="45" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="46" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="47" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="48" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="49" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="50" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="51" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="52" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="53" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="54" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="55" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="56" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="57" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="58" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="59" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="60" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="61" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="62" spans="2:2" ht="14.25" customHeight="1">
       <c r="B62" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="63" ht="14.25" customHeight="1">
+    <row r="63" spans="2:2" ht="14.25" customHeight="1">
       <c r="B63" s="4"/>
     </row>
-    <row r="64" ht="14.25" customHeight="1">
+    <row r="64" spans="2:2" ht="14.25" customHeight="1">
       <c r="B64" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="65" ht="14.25" customHeight="1">
+    <row r="65" spans="2:2" ht="14.25" customHeight="1">
       <c r="B65" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="66" ht="14.25" customHeight="1">
+    <row r="66" spans="2:2" ht="14.25" customHeight="1">
       <c r="B66" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="67" ht="14.25" customHeight="1">
+    <row r="67" spans="2:2" ht="14.25" customHeight="1">
       <c r="B67" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="68" ht="14.25" customHeight="1"/>
-    <row r="69" ht="14.25" customHeight="1"/>
-    <row r="70" ht="14.25" customHeight="1"/>
-    <row r="71" ht="14.25" customHeight="1"/>
-    <row r="72" ht="14.25" customHeight="1"/>
-    <row r="73" ht="14.25" customHeight="1"/>
-    <row r="74" ht="14.25" customHeight="1"/>
-    <row r="75" ht="14.25" customHeight="1"/>
-    <row r="76" ht="14.25" customHeight="1"/>
-    <row r="77" ht="14.25" customHeight="1"/>
-    <row r="78" ht="14.25" customHeight="1"/>
-    <row r="79" ht="14.25" customHeight="1"/>
-    <row r="80" ht="14.25" customHeight="1"/>
-    <row r="81" ht="14.25" customHeight="1"/>
-    <row r="82" ht="14.25" customHeight="1"/>
-    <row r="83" ht="14.25" customHeight="1"/>
-    <row r="84" ht="14.25" customHeight="1"/>
-    <row r="85" ht="14.25" customHeight="1"/>
-    <row r="86" ht="14.25" customHeight="1"/>
-    <row r="87" ht="14.25" customHeight="1"/>
-    <row r="88" ht="14.25" customHeight="1"/>
-    <row r="89" ht="14.25" customHeight="1">
+    <row r="68" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="69" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="70" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="71" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="72" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="73" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="74" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="75" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="76" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="77" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="78" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="79" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="80" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="81" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="82" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="83" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="84" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="85" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="86" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="87" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="88" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="89" spans="2:2" ht="14.25" customHeight="1">
       <c r="B89" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="90" ht="14.25" customHeight="1"/>
-    <row r="91" ht="14.25" customHeight="1">
+    <row r="90" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="91" spans="2:2" ht="14.25" customHeight="1">
       <c r="B91" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="92" ht="14.25" customHeight="1">
+    <row r="92" spans="2:2" ht="14.25" customHeight="1">
       <c r="B92" s="5"/>
     </row>
-    <row r="93" ht="14.25" customHeight="1">
+    <row r="93" spans="2:2" ht="14.25" customHeight="1">
       <c r="B93" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="94" ht="14.25" customHeight="1">
+    <row r="94" spans="2:2" ht="14.25" customHeight="1">
       <c r="B94" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="95" ht="14.25" customHeight="1">
+    <row r="95" spans="2:2" ht="14.25" customHeight="1">
       <c r="B95" s="6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="96" ht="14.25" customHeight="1"/>
-    <row r="97" ht="14.25" customHeight="1">
-      <c r="B97" s="2" t="s">
+    <row r="96" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B96" s="11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="97" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="98" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B98" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="98" ht="14.25" customHeight="1"/>
-    <row r="99" ht="14.25" customHeight="1"/>
-    <row r="100" ht="14.25" customHeight="1"/>
-    <row r="101" ht="14.25" customHeight="1"/>
-    <row r="102" ht="14.25" customHeight="1"/>
-    <row r="103" ht="14.25" customHeight="1"/>
-    <row r="104" ht="14.25" customHeight="1"/>
-    <row r="105" ht="14.25" customHeight="1"/>
-    <row r="106" ht="14.25" customHeight="1"/>
-    <row r="107" ht="14.25" customHeight="1"/>
-    <row r="108" ht="14.25" customHeight="1"/>
-    <row r="109" ht="14.25" customHeight="1"/>
-    <row r="110" ht="14.25" customHeight="1"/>
-    <row r="111" ht="14.25" customHeight="1"/>
-    <row r="112" ht="14.25" customHeight="1"/>
-    <row r="113" ht="14.25" customHeight="1"/>
-    <row r="114" ht="14.25" customHeight="1"/>
-    <row r="115" ht="14.25" customHeight="1"/>
-    <row r="116" ht="14.25" customHeight="1"/>
-    <row r="117" ht="14.25" customHeight="1"/>
-    <row r="118" ht="14.25" customHeight="1"/>
-    <row r="119" ht="14.25" customHeight="1">
-      <c r="B119" s="3" t="s">
+    <row r="99" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="100" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="101" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="102" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="103" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="104" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="105" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="106" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="107" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="108" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="109" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="110" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="111" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="112" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="113" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="114" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="115" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="116" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="117" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="118" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="119" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="120" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B120" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="120" ht="14.25" customHeight="1"/>
-    <row r="121" ht="14.25" customHeight="1">
-      <c r="B121" s="2" t="s">
+    <row r="121" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="122" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B122" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="122" ht="14.25" customHeight="1"/>
-    <row r="123" ht="14.25" customHeight="1">
-      <c r="B123" s="7" t="s">
+    <row r="123" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="124" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B124" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="124" ht="14.25" customHeight="1"/>
-    <row r="125" ht="14.25" customHeight="1"/>
-    <row r="126" ht="14.25" customHeight="1"/>
-    <row r="127" ht="14.25" customHeight="1"/>
-    <row r="128" ht="14.25" customHeight="1"/>
+    <row r="125" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="126" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="127" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="128" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="129" ht="14.25" customHeight="1"/>
     <row r="130" ht="14.25" customHeight="1"/>
     <row r="131" ht="14.25" customHeight="1"/>
@@ -1819,77 +1873,77 @@
     <row r="142" ht="14.25" customHeight="1"/>
     <row r="143" ht="14.25" customHeight="1"/>
     <row r="144" ht="14.25" customHeight="1"/>
-    <row r="145" ht="14.25" customHeight="1">
-      <c r="B145" s="3" t="s">
+    <row r="145" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="146" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B146" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="146" ht="14.25" customHeight="1">
-      <c r="B146" s="4"/>
-    </row>
-    <row r="147" ht="14.25" customHeight="1">
-      <c r="B147" s="4" t="s">
+    <row r="147" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B147" s="4"/>
+    </row>
+    <row r="148" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B148" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="148" ht="14.25" customHeight="1">
-      <c r="B148" s="4"/>
-    </row>
-    <row r="149" ht="14.25" customHeight="1">
-      <c r="B149" s="8" t="s">
+    <row r="149" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B149" s="4"/>
+    </row>
+    <row r="150" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B150" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="Q149" s="2" t="s">
+      <c r="Q150" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="150" ht="14.25" customHeight="1">
-      <c r="B150" s="8" t="s">
+    <row r="151" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B151" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="Q150" s="8" t="s">
+      <c r="Q151" s="8" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="151" ht="14.25" customHeight="1"/>
-    <row r="152" ht="14.25" customHeight="1"/>
-    <row r="153" ht="14.25" customHeight="1"/>
-    <row r="154" ht="14.25" customHeight="1"/>
-    <row r="155" ht="14.25" customHeight="1"/>
-    <row r="156" ht="14.25" customHeight="1"/>
-    <row r="157" ht="14.25" customHeight="1"/>
-    <row r="158" ht="14.25" customHeight="1"/>
-    <row r="159" ht="14.25" customHeight="1"/>
-    <row r="160" ht="14.25" customHeight="1"/>
-    <row r="161" ht="14.25" customHeight="1"/>
-    <row r="162" ht="14.25" customHeight="1"/>
-    <row r="163" ht="14.25" customHeight="1"/>
-    <row r="164" ht="14.25" customHeight="1"/>
-    <row r="165" ht="14.25" customHeight="1"/>
-    <row r="166" ht="14.25" customHeight="1"/>
-    <row r="167" ht="14.25" customHeight="1"/>
-    <row r="168" ht="14.25" customHeight="1"/>
-    <row r="169" ht="14.25" customHeight="1"/>
-    <row r="170" ht="14.25" customHeight="1"/>
-    <row r="171" ht="14.25" customHeight="1"/>
-    <row r="172" ht="14.25" customHeight="1"/>
-    <row r="173" ht="14.25" customHeight="1">
-      <c r="B173" s="4"/>
-    </row>
-    <row r="174" ht="14.25" customHeight="1">
-      <c r="B174" s="8" t="s">
+    <row r="152" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="153" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="154" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="155" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="156" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="157" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="158" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="159" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="160" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="161" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="162" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="163" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="164" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="165" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="166" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="167" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="168" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="169" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="170" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="171" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="172" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="173" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="174" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B174" s="4"/>
+    </row>
+    <row r="175" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B175" s="8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="175" ht="14.25" customHeight="1">
-      <c r="B175" s="8" t="s">
+    <row r="176" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B176" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="Q175" s="8" t="s">
+      <c r="Q176" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="176" ht="14.25" customHeight="1"/>
     <row r="177" ht="14.25" customHeight="1"/>
     <row r="178" ht="14.25" customHeight="1"/>
     <row r="179" ht="14.25" customHeight="1"/>
@@ -1906,33 +1960,33 @@
     <row r="190" ht="14.25" customHeight="1"/>
     <row r="191" ht="14.25" customHeight="1"/>
     <row r="192" ht="14.25" customHeight="1"/>
-    <row r="193" ht="14.25" customHeight="1"/>
-    <row r="194" ht="14.25" customHeight="1"/>
-    <row r="195" ht="14.25" customHeight="1"/>
-    <row r="196" ht="14.25" customHeight="1"/>
-    <row r="197" ht="14.25" customHeight="1"/>
-    <row r="198" ht="14.25" customHeight="1"/>
-    <row r="199" ht="14.25" customHeight="1">
-      <c r="B199" s="8" t="s">
+    <row r="193" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="194" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="195" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="196" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="197" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="198" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="199" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="200" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B200" s="8" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="200" ht="14.25" customHeight="1">
-      <c r="B200" s="8" t="s">
+    <row r="201" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B201" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="Q200" s="8" t="s">
+      <c r="Q201" s="8" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="201" ht="14.25" customHeight="1"/>
-    <row r="202" ht="14.25" customHeight="1"/>
-    <row r="203" ht="14.25" customHeight="1"/>
-    <row r="204" ht="14.25" customHeight="1"/>
-    <row r="205" ht="14.25" customHeight="1"/>
-    <row r="206" ht="14.25" customHeight="1"/>
-    <row r="207" ht="14.25" customHeight="1"/>
-    <row r="208" ht="14.25" customHeight="1"/>
+    <row r="202" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="203" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="204" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="205" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="206" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="207" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="208" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="209" ht="14.25" customHeight="1"/>
     <row r="210" ht="14.25" customHeight="1"/>
     <row r="211" ht="14.25" customHeight="1"/>
@@ -1949,266 +2003,266 @@
     <row r="222" ht="14.25" customHeight="1"/>
     <row r="223" ht="14.25" customHeight="1"/>
     <row r="224" ht="14.25" customHeight="1"/>
-    <row r="225" ht="14.25" customHeight="1">
-      <c r="B225" s="3" t="s">
+    <row r="225" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="226" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B226" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="226" ht="14.25" customHeight="1">
-      <c r="B226" s="4"/>
-    </row>
-    <row r="227" ht="14.25" customHeight="1">
-      <c r="B227" s="4" t="s">
+    <row r="227" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B227" s="4"/>
+    </row>
+    <row r="228" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B228" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="228" ht="14.25" customHeight="1">
-      <c r="B228" s="9" t="s">
+    <row r="229" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B229" s="9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="229" ht="14.25" customHeight="1">
-      <c r="B229" s="9" t="s">
+    <row r="230" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B230" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="230" ht="14.25" customHeight="1"/>
-    <row r="231" ht="14.25" customHeight="1"/>
-    <row r="232" ht="14.25" customHeight="1"/>
-    <row r="233" ht="14.25" customHeight="1"/>
-    <row r="234" ht="14.25" customHeight="1"/>
-    <row r="235" ht="14.25" customHeight="1"/>
-    <row r="236" ht="14.25" customHeight="1"/>
-    <row r="237" ht="14.25" customHeight="1"/>
-    <row r="238" ht="14.25" customHeight="1"/>
-    <row r="239" ht="14.25" customHeight="1"/>
-    <row r="240" ht="14.25" customHeight="1"/>
-    <row r="241" ht="14.25" customHeight="1"/>
-    <row r="242" ht="14.25" customHeight="1"/>
-    <row r="243" ht="14.25" customHeight="1"/>
-    <row r="244" ht="14.25" customHeight="1"/>
-    <row r="245" ht="14.25" customHeight="1"/>
-    <row r="246" ht="14.25" customHeight="1"/>
-    <row r="247" ht="14.25" customHeight="1"/>
-    <row r="248" ht="14.25" customHeight="1"/>
-    <row r="249" ht="14.25" customHeight="1"/>
-    <row r="250" ht="14.25" customHeight="1"/>
-    <row r="251" ht="14.25" customHeight="1">
-      <c r="B251" s="3" t="s">
+    <row r="231" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="232" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="233" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="234" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="235" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="236" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="237" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="238" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="239" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="240" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="241" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="242" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="243" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="244" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="245" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="246" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="247" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="248" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="249" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="250" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="251" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="252" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B252" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="252" ht="14.25" customHeight="1"/>
-    <row r="253" ht="14.25" customHeight="1">
-      <c r="B253" s="2" t="s">
+    <row r="253" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="254" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B254" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="254" ht="14.25" customHeight="1">
-      <c r="B254" s="4"/>
-    </row>
-    <row r="255" ht="14.25" customHeight="1">
-      <c r="B255" s="10" t="s">
+    <row r="255" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B255" s="4"/>
+    </row>
+    <row r="256" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B256" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="256" ht="14.25" customHeight="1">
-      <c r="B256" s="4" t="s">
+    <row r="257" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B257" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="257" ht="14.25" customHeight="1">
-      <c r="B257" s="9" t="s">
+    <row r="258" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B258" s="9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="258" ht="14.25" customHeight="1">
-      <c r="B258" s="4"/>
-    </row>
-    <row r="259" ht="14.25" customHeight="1">
+    <row r="259" spans="2:2" ht="14.25" customHeight="1">
       <c r="B259" s="4"/>
     </row>
-    <row r="260" ht="14.25" customHeight="1">
+    <row r="260" spans="2:2" ht="14.25" customHeight="1">
       <c r="B260" s="4"/>
     </row>
-    <row r="261" ht="14.25" customHeight="1">
+    <row r="261" spans="2:2" ht="14.25" customHeight="1">
       <c r="B261" s="4"/>
     </row>
-    <row r="262" ht="14.25" customHeight="1">
+    <row r="262" spans="2:2" ht="14.25" customHeight="1">
       <c r="B262" s="4"/>
     </row>
-    <row r="263" ht="14.25" customHeight="1">
+    <row r="263" spans="2:2" ht="14.25" customHeight="1">
       <c r="B263" s="4"/>
     </row>
-    <row r="264" ht="14.25" customHeight="1">
+    <row r="264" spans="2:2" ht="14.25" customHeight="1">
       <c r="B264" s="4"/>
     </row>
-    <row r="265" ht="14.25" customHeight="1">
+    <row r="265" spans="2:2" ht="14.25" customHeight="1">
       <c r="B265" s="4"/>
     </row>
-    <row r="266" ht="14.25" customHeight="1">
+    <row r="266" spans="2:2" ht="14.25" customHeight="1">
       <c r="B266" s="4"/>
     </row>
-    <row r="267" ht="14.25" customHeight="1">
+    <row r="267" spans="2:2" ht="14.25" customHeight="1">
       <c r="B267" s="4"/>
     </row>
-    <row r="268" ht="14.25" customHeight="1">
+    <row r="268" spans="2:2" ht="14.25" customHeight="1">
       <c r="B268" s="4"/>
     </row>
-    <row r="269" ht="14.25" customHeight="1">
+    <row r="269" spans="2:2" ht="14.25" customHeight="1">
       <c r="B269" s="4"/>
     </row>
-    <row r="270" ht="14.25" customHeight="1">
+    <row r="270" spans="2:2" ht="14.25" customHeight="1">
       <c r="B270" s="4"/>
     </row>
-    <row r="271" ht="14.25" customHeight="1">
+    <row r="271" spans="2:2" ht="14.25" customHeight="1">
       <c r="B271" s="4"/>
     </row>
-    <row r="272" ht="14.25" customHeight="1">
+    <row r="272" spans="2:2" ht="14.25" customHeight="1">
       <c r="B272" s="4"/>
     </row>
-    <row r="273" ht="14.25" customHeight="1">
+    <row r="273" spans="2:2" ht="14.25" customHeight="1">
       <c r="B273" s="4"/>
     </row>
-    <row r="274" ht="14.25" customHeight="1">
+    <row r="274" spans="2:2" ht="14.25" customHeight="1">
       <c r="B274" s="4"/>
     </row>
-    <row r="275" ht="14.25" customHeight="1">
+    <row r="275" spans="2:2" ht="14.25" customHeight="1">
       <c r="B275" s="4"/>
     </row>
-    <row r="276" ht="14.25" customHeight="1">
+    <row r="276" spans="2:2" ht="14.25" customHeight="1">
       <c r="B276" s="4"/>
     </row>
-    <row r="277" ht="14.25" customHeight="1">
+    <row r="277" spans="2:2" ht="14.25" customHeight="1">
       <c r="B277" s="4"/>
     </row>
-    <row r="278" ht="14.25" customHeight="1">
+    <row r="278" spans="2:2" ht="14.25" customHeight="1">
       <c r="B278" s="4"/>
     </row>
-    <row r="279" ht="14.25" customHeight="1">
+    <row r="279" spans="2:2" ht="14.25" customHeight="1">
       <c r="B279" s="4"/>
     </row>
-    <row r="280" ht="14.25" customHeight="1">
+    <row r="280" spans="2:2" ht="14.25" customHeight="1">
       <c r="B280" s="4"/>
     </row>
-    <row r="281" ht="14.25" customHeight="1">
+    <row r="281" spans="2:2" ht="14.25" customHeight="1">
       <c r="B281" s="4"/>
     </row>
-    <row r="282" ht="14.25" customHeight="1">
+    <row r="282" spans="2:2" ht="14.25" customHeight="1">
       <c r="B282" s="4"/>
     </row>
-    <row r="283" ht="14.25" customHeight="1">
+    <row r="283" spans="2:2" ht="14.25" customHeight="1">
       <c r="B283" s="4"/>
     </row>
-    <row r="284" ht="14.25" customHeight="1">
-      <c r="B284" s="10" t="s">
+    <row r="284" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B284" s="4"/>
+    </row>
+    <row r="285" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B285" s="10" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="285" ht="14.25" customHeight="1">
-      <c r="B285" s="4" t="s">
+    <row r="286" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B286" s="4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="286" ht="14.25" customHeight="1">
-      <c r="B286" s="4"/>
-    </row>
-    <row r="287" ht="14.25" customHeight="1">
+    <row r="287" spans="2:2" ht="14.25" customHeight="1">
       <c r="B287" s="4"/>
     </row>
-    <row r="288" ht="14.25" customHeight="1">
+    <row r="288" spans="2:2" ht="14.25" customHeight="1">
       <c r="B288" s="4"/>
     </row>
-    <row r="289" ht="14.25" customHeight="1">
+    <row r="289" spans="2:2" ht="14.25" customHeight="1">
       <c r="B289" s="4"/>
     </row>
-    <row r="290" ht="14.25" customHeight="1">
+    <row r="290" spans="2:2" ht="14.25" customHeight="1">
       <c r="B290" s="4"/>
     </row>
-    <row r="291" ht="14.25" customHeight="1">
+    <row r="291" spans="2:2" ht="14.25" customHeight="1">
       <c r="B291" s="4"/>
     </row>
-    <row r="292" ht="14.25" customHeight="1">
+    <row r="292" spans="2:2" ht="14.25" customHeight="1">
       <c r="B292" s="4"/>
     </row>
-    <row r="293" ht="14.25" customHeight="1">
+    <row r="293" spans="2:2" ht="14.25" customHeight="1">
       <c r="B293" s="4"/>
     </row>
-    <row r="294" ht="14.25" customHeight="1">
+    <row r="294" spans="2:2" ht="14.25" customHeight="1">
       <c r="B294" s="4"/>
     </row>
-    <row r="295" ht="14.25" customHeight="1">
+    <row r="295" spans="2:2" ht="14.25" customHeight="1">
       <c r="B295" s="4"/>
     </row>
-    <row r="296" ht="14.25" customHeight="1">
+    <row r="296" spans="2:2" ht="14.25" customHeight="1">
       <c r="B296" s="4"/>
     </row>
-    <row r="297" ht="14.25" customHeight="1">
+    <row r="297" spans="2:2" ht="14.25" customHeight="1">
       <c r="B297" s="4"/>
     </row>
-    <row r="298" ht="14.25" customHeight="1">
+    <row r="298" spans="2:2" ht="14.25" customHeight="1">
       <c r="B298" s="4"/>
     </row>
-    <row r="299" ht="14.25" customHeight="1">
+    <row r="299" spans="2:2" ht="14.25" customHeight="1">
       <c r="B299" s="4"/>
     </row>
-    <row r="300" ht="14.25" customHeight="1">
+    <row r="300" spans="2:2" ht="14.25" customHeight="1">
       <c r="B300" s="4"/>
     </row>
-    <row r="301" ht="14.25" customHeight="1">
+    <row r="301" spans="2:2" ht="14.25" customHeight="1">
       <c r="B301" s="4"/>
     </row>
-    <row r="302" ht="14.25" customHeight="1">
+    <row r="302" spans="2:2" ht="14.25" customHeight="1">
       <c r="B302" s="4"/>
     </row>
-    <row r="303" ht="14.25" customHeight="1">
+    <row r="303" spans="2:2" ht="14.25" customHeight="1">
       <c r="B303" s="4"/>
     </row>
-    <row r="304" ht="14.25" customHeight="1">
+    <row r="304" spans="2:2" ht="14.25" customHeight="1">
       <c r="B304" s="4"/>
     </row>
-    <row r="305" ht="14.25" customHeight="1">
+    <row r="305" spans="2:2" ht="14.25" customHeight="1">
       <c r="B305" s="4"/>
     </row>
-    <row r="306" ht="14.25" customHeight="1">
+    <row r="306" spans="2:2" ht="14.25" customHeight="1">
       <c r="B306" s="4"/>
     </row>
-    <row r="307" ht="14.25" customHeight="1">
+    <row r="307" spans="2:2" ht="14.25" customHeight="1">
       <c r="B307" s="4"/>
     </row>
-    <row r="308" ht="14.25" customHeight="1">
+    <row r="308" spans="2:2" ht="14.25" customHeight="1">
       <c r="B308" s="4"/>
     </row>
-    <row r="309" ht="14.25" customHeight="1">
+    <row r="309" spans="2:2" ht="14.25" customHeight="1">
       <c r="B309" s="4"/>
     </row>
-    <row r="310" ht="14.25" customHeight="1">
+    <row r="310" spans="2:2" ht="14.25" customHeight="1">
       <c r="B310" s="4"/>
     </row>
-    <row r="311" ht="14.25" customHeight="1">
+    <row r="311" spans="2:2" ht="14.25" customHeight="1">
       <c r="B311" s="4"/>
     </row>
-    <row r="312" ht="14.25" customHeight="1">
+    <row r="312" spans="2:2" ht="14.25" customHeight="1">
       <c r="B312" s="4"/>
     </row>
-    <row r="313" ht="14.25" customHeight="1">
+    <row r="313" spans="2:2" ht="14.25" customHeight="1">
       <c r="B313" s="4"/>
     </row>
-    <row r="314" ht="14.25" customHeight="1">
-      <c r="B314" s="10" t="s">
+    <row r="314" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B314" s="4"/>
+    </row>
+    <row r="315" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B315" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="315" ht="14.25" customHeight="1">
-      <c r="B315" s="4" t="s">
+    <row r="316" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B316" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="316" ht="14.25" customHeight="1"/>
-    <row r="317" ht="14.25" customHeight="1"/>
-    <row r="318" ht="14.25" customHeight="1"/>
-    <row r="319" ht="14.25" customHeight="1"/>
-    <row r="320" ht="14.25" customHeight="1"/>
+    <row r="317" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="318" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="319" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="320" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="321" ht="14.25" customHeight="1"/>
     <row r="322" ht="14.25" customHeight="1"/>
     <row r="323" ht="14.25" customHeight="1"/>
@@ -2225,40 +2279,40 @@
     <row r="334" ht="14.25" customHeight="1"/>
     <row r="335" ht="14.25" customHeight="1"/>
     <row r="336" ht="14.25" customHeight="1"/>
-    <row r="337" ht="14.25" customHeight="1"/>
-    <row r="338" ht="14.25" customHeight="1"/>
-    <row r="339" ht="14.25" customHeight="1"/>
-    <row r="340" ht="14.25" customHeight="1"/>
-    <row r="341" ht="14.25" customHeight="1"/>
-    <row r="342" ht="14.25" customHeight="1">
-      <c r="B342" s="3" t="s">
+    <row r="337" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="338" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="339" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="340" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="341" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="342" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="343" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B343" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="343" ht="14.25" customHeight="1">
-      <c r="B343" s="4"/>
-    </row>
-    <row r="344" ht="14.25" customHeight="1">
-      <c r="B344" s="9" t="s">
+    <row r="344" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B344" s="4"/>
+    </row>
+    <row r="345" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B345" s="9" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="345" ht="14.25" customHeight="1">
-      <c r="B345" s="4" t="s">
+    <row r="346" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B346" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="346" ht="14.25" customHeight="1">
-      <c r="B346" s="4" t="s">
+    <row r="347" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B347" s="4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="347" ht="14.25" customHeight="1"/>
-    <row r="348" ht="14.25" customHeight="1"/>
-    <row r="349" ht="14.25" customHeight="1"/>
-    <row r="350" ht="14.25" customHeight="1"/>
-    <row r="351" ht="14.25" customHeight="1"/>
-    <row r="352" ht="14.25" customHeight="1"/>
+    <row r="348" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="349" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="350" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="351" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="352" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="353" ht="14.25" customHeight="1"/>
     <row r="354" ht="14.25" customHeight="1"/>
     <row r="355" ht="14.25" customHeight="1"/>
@@ -2275,42 +2329,42 @@
     <row r="366" ht="14.25" customHeight="1"/>
     <row r="367" ht="14.25" customHeight="1"/>
     <row r="368" ht="14.25" customHeight="1"/>
-    <row r="369" ht="14.25" customHeight="1"/>
-    <row r="370" ht="14.25" customHeight="1"/>
-    <row r="371" ht="14.25" customHeight="1"/>
-    <row r="372" ht="14.25" customHeight="1">
-      <c r="B372" s="2" t="s">
+    <row r="369" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="370" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="371" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="372" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="373" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B373" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="373" ht="14.25" customHeight="1"/>
-    <row r="374" ht="14.25" customHeight="1">
-      <c r="B374" s="3" t="s">
+    <row r="374" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="375" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B375" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="375" ht="14.25" customHeight="1">
-      <c r="B375" s="4"/>
-    </row>
-    <row r="376" ht="14.25" customHeight="1">
-      <c r="B376" s="4" t="s">
+    <row r="376" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B376" s="4"/>
+    </row>
+    <row r="377" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B377" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="377" ht="14.25" customHeight="1">
-      <c r="B377" s="9" t="s">
+    <row r="378" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B378" s="9" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="378" ht="14.25" customHeight="1">
-      <c r="B378" s="4"/>
-    </row>
-    <row r="379" ht="14.25" customHeight="1"/>
-    <row r="380" ht="14.25" customHeight="1"/>
-    <row r="381" ht="14.25" customHeight="1"/>
-    <row r="382" ht="14.25" customHeight="1"/>
-    <row r="383" ht="14.25" customHeight="1"/>
-    <row r="384" ht="14.25" customHeight="1"/>
+    <row r="379" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B379" s="4"/>
+    </row>
+    <row r="380" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="381" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="382" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="383" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="384" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="385" ht="14.25" customHeight="1"/>
     <row r="386" ht="14.25" customHeight="1"/>
     <row r="387" ht="14.25" customHeight="1"/>
@@ -2327,40 +2381,40 @@
     <row r="398" ht="14.25" customHeight="1"/>
     <row r="399" ht="14.25" customHeight="1"/>
     <row r="400" ht="14.25" customHeight="1"/>
-    <row r="401" ht="14.25" customHeight="1"/>
-    <row r="402" ht="14.25" customHeight="1"/>
-    <row r="403" ht="14.25" customHeight="1"/>
-    <row r="404" ht="14.25" customHeight="1"/>
-    <row r="405" ht="14.25" customHeight="1"/>
-    <row r="406" ht="14.25" customHeight="1">
-      <c r="B406" s="3" t="s">
+    <row r="401" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="402" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="403" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="404" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="405" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="406" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="407" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B407" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="407" ht="14.25" customHeight="1">
-      <c r="B407" s="4"/>
-    </row>
-    <row r="408" ht="14.25" customHeight="1">
-      <c r="B408" s="4" t="s">
+    <row r="408" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B408" s="4"/>
+    </row>
+    <row r="409" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B409" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="409" ht="14.25" customHeight="1">
-      <c r="B409" s="4" t="s">
+    <row r="410" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B410" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="410" ht="14.25" customHeight="1">
-      <c r="B410" s="4" t="s">
+    <row r="411" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B411" s="4" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="411" ht="14.25" customHeight="1"/>
-    <row r="412" ht="14.25" customHeight="1"/>
-    <row r="413" ht="14.25" customHeight="1"/>
-    <row r="414" ht="14.25" customHeight="1"/>
-    <row r="415" ht="14.25" customHeight="1"/>
-    <row r="416" ht="14.25" customHeight="1"/>
+    <row r="412" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="413" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="414" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="415" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="416" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="417" ht="14.25" customHeight="1"/>
     <row r="418" ht="14.25" customHeight="1"/>
     <row r="419" ht="14.25" customHeight="1"/>
@@ -2948,9 +3002,9 @@
     <row r="1001" ht="14.25" customHeight="1"/>
     <row r="1002" ht="14.25" customHeight="1"/>
     <row r="1003" ht="14.25" customHeight="1"/>
+    <row r="1004" ht="14.25" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: connection sheet added.
</commit_message>
<xml_diff>
--- a/SmartBU/How_To_Debugg.xlsx
+++ b/SmartBU/How_To_Debugg.xlsx
@@ -9,12 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9070" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9070" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Revision_1.0" sheetId="1" r:id="rId1"/>
     <sheet name="Revision_1.1" sheetId="2" r:id="rId2"/>
-    <sheet name="Connection" sheetId="3" r:id="rId3"/>
+    <sheet name="Connection " sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="189">
   <si>
     <t>Project Setup Using Trace32</t>
   </si>
@@ -632,9 +632,6 @@
     <t xml:space="preserve">LIN </t>
   </si>
   <si>
-    <t>Capa Singal Dip Switch</t>
-  </si>
-  <si>
     <t>Capa</t>
   </si>
   <si>
@@ -778,16 +775,287 @@
   <si>
     <t>4. Select the variant according to your connected hardware.</t>
   </si>
+  <si>
+    <t>Capa Singal Dip Switch 100pF</t>
+  </si>
+  <si>
+    <t>S.NO</t>
+  </si>
+  <si>
+    <t>Test Point</t>
+  </si>
+  <si>
+    <t>Signal Name</t>
+  </si>
+  <si>
+    <t>IDC Connector pin</t>
+  </si>
+  <si>
+    <t>TP100</t>
+  </si>
+  <si>
+    <t>12V</t>
+  </si>
+  <si>
+    <t>PIN 1</t>
+  </si>
+  <si>
+    <t>TP101</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>PIN 2</t>
+  </si>
+  <si>
+    <t>TP113</t>
+  </si>
+  <si>
+    <t>3V3</t>
+  </si>
+  <si>
+    <t>PIN 3</t>
+  </si>
+  <si>
+    <t>TP123</t>
+  </si>
+  <si>
+    <t>3V8</t>
+  </si>
+  <si>
+    <t>PIN 4</t>
+  </si>
+  <si>
+    <t>TP307</t>
+  </si>
+  <si>
+    <t>SG Power switch</t>
+  </si>
+  <si>
+    <t>PIN 5</t>
+  </si>
+  <si>
+    <t>TP310</t>
+  </si>
+  <si>
+    <t>SG1 op-amp output</t>
+  </si>
+  <si>
+    <t>PIN 6</t>
+  </si>
+  <si>
+    <t>TP311</t>
+  </si>
+  <si>
+    <t>SG1 IN1+ Input</t>
+  </si>
+  <si>
+    <t>PIN 7</t>
+  </si>
+  <si>
+    <t>TP312</t>
+  </si>
+  <si>
+    <t>SG1 IN1- Input</t>
+  </si>
+  <si>
+    <t>PIN 8</t>
+  </si>
+  <si>
+    <t>TP321</t>
+  </si>
+  <si>
+    <t>SG2 op-amp output</t>
+  </si>
+  <si>
+    <t>PIN 9</t>
+  </si>
+  <si>
+    <t>TP322</t>
+  </si>
+  <si>
+    <t>SG2 IN2+ Input</t>
+  </si>
+  <si>
+    <t>PIN 10</t>
+  </si>
+  <si>
+    <t>TP324</t>
+  </si>
+  <si>
+    <t>SG2 IN2- Input</t>
+  </si>
+  <si>
+    <t>PIN 11</t>
+  </si>
+  <si>
+    <t>TP407</t>
+  </si>
+  <si>
+    <t>AI_MOTOR_VISEN</t>
+  </si>
+  <si>
+    <t>PIN 12</t>
+  </si>
+  <si>
+    <t>DRV_OUT_A</t>
+  </si>
+  <si>
+    <t>Actuator</t>
+  </si>
+  <si>
+    <t>DB9 Conn</t>
+  </si>
+  <si>
+    <t>DRV_OUT_B</t>
+  </si>
+  <si>
+    <t>TP414</t>
+  </si>
+  <si>
+    <t>AI_MOTOR_DIAG</t>
+  </si>
+  <si>
+    <t>PIN 15</t>
+  </si>
+  <si>
+    <t>TP503</t>
+  </si>
+  <si>
+    <t>Cap Unlock pin</t>
+  </si>
+  <si>
+    <t>PIN 16</t>
+  </si>
+  <si>
+    <t>TP505</t>
+  </si>
+  <si>
+    <t>Cap Unlock reference</t>
+  </si>
+  <si>
+    <t>PIN 17</t>
+  </si>
+  <si>
+    <t>TP507</t>
+  </si>
+  <si>
+    <t>Cap proximity</t>
+  </si>
+  <si>
+    <t>PIN 18</t>
+  </si>
+  <si>
+    <t>TP509</t>
+  </si>
+  <si>
+    <t>Cap proximity reference</t>
+  </si>
+  <si>
+    <t>PIN 19</t>
+  </si>
+  <si>
+    <t>TP511</t>
+  </si>
+  <si>
+    <t>Cap lock</t>
+  </si>
+  <si>
+    <t>PIN 20</t>
+  </si>
+  <si>
+    <t>TP602</t>
+  </si>
+  <si>
+    <t>Led out pin</t>
+  </si>
+  <si>
+    <t>PIN 21</t>
+  </si>
+  <si>
+    <t>TP612</t>
+  </si>
+  <si>
+    <t>AI_EOS_DIAG</t>
+  </si>
+  <si>
+    <t>PIN 22</t>
+  </si>
+  <si>
+    <t>TP613</t>
+  </si>
+  <si>
+    <t>EOS_Out</t>
+  </si>
+  <si>
+    <t>PIN 23</t>
+  </si>
+  <si>
+    <t>TP614</t>
+  </si>
+  <si>
+    <t>IPB GND</t>
+  </si>
+  <si>
+    <t>PIN 24</t>
+  </si>
+  <si>
+    <t>TP104</t>
+  </si>
+  <si>
+    <t>PIN 25</t>
+  </si>
+  <si>
+    <t>TP106</t>
+  </si>
+  <si>
+    <t>PIN 26</t>
+  </si>
+  <si>
+    <t>TP200</t>
+  </si>
+  <si>
+    <t>RESET</t>
+  </si>
+  <si>
+    <t>PIN 29</t>
+  </si>
+  <si>
+    <t>TP201</t>
+  </si>
+  <si>
+    <t>SWD_DATA</t>
+  </si>
+  <si>
+    <t>PIN 27</t>
+  </si>
+  <si>
+    <t>TP202</t>
+  </si>
+  <si>
+    <t>SWD_CLK</t>
+  </si>
+  <si>
+    <t>PIN 28</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -938,79 +1206,91 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 3" xfId="3"/>
     <cellStyle name="標準 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2526,14 +2806,19 @@
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>7620</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>165169</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="5456518" cy="3951274"/>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>585843</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Picture 1"/>
@@ -2550,7 +2835,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1226820" y="5873819"/>
-          <a:ext cx="5456518" cy="3951274"/>
+          <a:ext cx="5442323" cy="3893751"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2558,15 +2843,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>580016</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>172219</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="5926069" cy="3911346"/>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>402614</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>161506</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Picture 2"/>
@@ -2583,7 +2873,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1799216" y="1461269"/>
-          <a:ext cx="5926069" cy="3911346"/>
+          <a:ext cx="5905898" cy="3856437"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2591,7 +2881,7 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
@@ -2607,7 +2897,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3985260" y="4196080"/>
+          <a:off x="4582160" y="4196080"/>
           <a:ext cx="262636" cy="468077"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2673,7 +2963,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2796540" y="4202004"/>
+          <a:off x="3368040" y="4202004"/>
           <a:ext cx="340606" cy="468077"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2739,7 +3029,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2956560" y="4585544"/>
+          <a:off x="3528060" y="4585544"/>
           <a:ext cx="1262653" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2808,7 +3098,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5006340" y="4617294"/>
+          <a:off x="5603240" y="4617294"/>
           <a:ext cx="851836" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2862,14 +3152,19 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>160020</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="3761776" cy="2607442"/>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>86247</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>152756</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="8" name="Picture 7"/>
@@ -2885,8 +3180,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="2553970"/>
-          <a:ext cx="3761776" cy="2607442"/>
+          <a:off x="8521700" y="2553970"/>
+          <a:ext cx="3743847" cy="2570836"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2894,7 +3189,7 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
@@ -2915,7 +3210,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3505200" y="4902200"/>
+          <a:off x="4102100" y="4902200"/>
           <a:ext cx="7620" cy="943610"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -2962,7 +3257,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="5981700" y="4434840"/>
+          <a:off x="6578600" y="4434840"/>
           <a:ext cx="1920240" cy="7620"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -3004,7 +3299,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9144000" y="2286000"/>
+          <a:off x="9740900" y="2286000"/>
           <a:ext cx="851836" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3058,14 +3353,19 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>367553</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>161364</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4901387" cy="5831014"/>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>368234</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>15908</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="12" name="Picture 11"/>
@@ -3081,8 +3381,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7073153" y="5870014"/>
-          <a:ext cx="4901387" cy="5831014"/>
+          <a:off x="7670053" y="5870014"/>
+          <a:ext cx="4877481" cy="5747344"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3090,7 +3390,7 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>15</xdr:col>
@@ -3106,7 +3406,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9305364" y="7559115"/>
+          <a:off x="9902264" y="7559115"/>
           <a:ext cx="262636" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3162,7 +3462,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10103222" y="7559115"/>
+          <a:off x="10700122" y="7559115"/>
           <a:ext cx="262636" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3218,7 +3518,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9663953" y="8699873"/>
+          <a:off x="10260853" y="8699873"/>
           <a:ext cx="262636" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3274,7 +3574,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10883153" y="9777880"/>
+          <a:off x="11480053" y="9777880"/>
           <a:ext cx="262636" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3330,7 +3630,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11376212" y="11120718"/>
+          <a:off x="11973112" y="11120718"/>
           <a:ext cx="262636" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3386,7 +3686,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8355106" y="10375152"/>
+          <a:off x="8952006" y="10375152"/>
           <a:ext cx="262636" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3442,7 +3742,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7682753" y="7199780"/>
+          <a:off x="8279653" y="7199780"/>
           <a:ext cx="262636" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3498,7 +3798,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8364071" y="6247280"/>
+          <a:off x="8960971" y="6247280"/>
           <a:ext cx="262636" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3554,7 +3854,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7261412" y="10927603"/>
+          <a:off x="7858312" y="10927603"/>
           <a:ext cx="340606" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3610,7 +3910,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7915835" y="9849597"/>
+          <a:off x="8512735" y="9849597"/>
           <a:ext cx="262636" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3666,7 +3966,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7924800" y="8726767"/>
+          <a:off x="8521700" y="8726767"/>
           <a:ext cx="340606" cy="280205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5761,7 +6061,7 @@
     </row>
     <row r="231" spans="2:2" ht="14.25" customHeight="1">
       <c r="B231" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="232" spans="2:2" ht="14.25" customHeight="1">
@@ -6132,19 +6432,19 @@
     <row r="409" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="410" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="411" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B411" s="19" t="s">
-        <v>96</v>
+      <c r="B411" s="12" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="412" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="413" spans="2:2" ht="14.25" customHeight="1">
       <c r="B413" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="414" spans="2:2" ht="14.25" customHeight="1">
       <c r="B414" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="415" spans="2:2" ht="14.25" customHeight="1"/>
@@ -6170,8 +6470,8 @@
     <row r="435" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="436" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="437" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B437" s="20" t="s">
-        <v>100</v>
+      <c r="B437" s="13" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="438" spans="2:2" ht="14.25" customHeight="1"/>
@@ -6197,8 +6497,8 @@
     <row r="458" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="459" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="460" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B460" s="20" t="s">
-        <v>101</v>
+      <c r="B460" s="13" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="461" spans="2:2" ht="14.25" customHeight="1"/>
@@ -6224,8 +6524,8 @@
     <row r="481" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="482" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="483" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B483" s="19" t="s">
-        <v>95</v>
+      <c r="B483" s="12" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="484" spans="2:2" ht="14.25" customHeight="1">
@@ -6848,289 +7148,929 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="C65:Q86"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <dimension ref="C65:Q116"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="3" width="8.81640625" style="12"/>
-    <col min="4" max="4" width="16.90625" style="12" customWidth="1"/>
-    <col min="5" max="5" width="9.08984375" style="12" customWidth="1"/>
-    <col min="6" max="16384" width="8.81640625" style="12"/>
+    <col min="1" max="3" width="8.7265625" style="14"/>
+    <col min="4" max="4" width="16.90625" style="14" customWidth="1"/>
+    <col min="5" max="5" width="9.08984375" style="14" customWidth="1"/>
+    <col min="6" max="16384" width="8.7265625" style="14"/>
   </cols>
   <sheetData>
     <row r="65" spans="3:17">
-      <c r="N65" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="O65" s="22"/>
-      <c r="P65" s="22"/>
-      <c r="Q65" s="22"/>
+      <c r="N65" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="O65" s="15"/>
+      <c r="P65" s="15"/>
+      <c r="Q65" s="15"/>
     </row>
     <row r="69" spans="3:17">
-      <c r="C69" s="23" t="s">
-        <v>93</v>
-      </c>
-      <c r="D69" s="23"/>
-      <c r="E69" s="23"/>
-      <c r="F69" s="23"/>
-      <c r="G69" s="23"/>
-      <c r="H69" s="23"/>
-      <c r="I69" s="23"/>
-      <c r="J69" s="23"/>
-      <c r="K69" s="23"/>
-      <c r="L69" s="23"/>
+      <c r="C69" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="D69" s="26"/>
+      <c r="E69" s="26"/>
+      <c r="F69" s="26"/>
+      <c r="G69" s="26"/>
+      <c r="H69" s="26"/>
+      <c r="I69" s="17"/>
+      <c r="J69" s="17"/>
+      <c r="K69" s="17"/>
+      <c r="L69" s="17"/>
     </row>
     <row r="70" spans="3:17">
       <c r="C70" s="18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D70" s="18" t="s">
-        <v>91</v>
-      </c>
-      <c r="E70" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="F70" s="24"/>
-      <c r="G70" s="24"/>
-      <c r="H70" s="24"/>
-      <c r="I70" s="15"/>
-      <c r="J70" s="15"/>
-      <c r="K70" s="15"/>
-      <c r="L70" s="15"/>
+      <c r="E70" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="F70" s="19"/>
+      <c r="G70" s="19"/>
+      <c r="H70" s="19"/>
+      <c r="I70" s="20"/>
+      <c r="J70" s="20"/>
+      <c r="K70" s="20"/>
+      <c r="L70" s="20"/>
     </row>
     <row r="71" spans="3:17">
-      <c r="C71" s="17">
+      <c r="C71" s="21">
         <v>1</v>
       </c>
-      <c r="D71" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="E71" s="21" t="s">
+      <c r="D71" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="F71" s="21"/>
-      <c r="G71" s="21"/>
-      <c r="H71" s="21"/>
-      <c r="I71" s="15"/>
-      <c r="J71" s="15"/>
-      <c r="K71" s="15"/>
-      <c r="L71" s="15"/>
+      <c r="E71" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="F71" s="16"/>
+      <c r="G71" s="16"/>
+      <c r="H71" s="16"/>
+      <c r="I71" s="20"/>
+      <c r="J71" s="20"/>
+      <c r="K71" s="20"/>
+      <c r="L71" s="20"/>
     </row>
     <row r="72" spans="3:17">
-      <c r="C72" s="17">
+      <c r="C72" s="21">
         <v>2</v>
       </c>
-      <c r="D72" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="E72" s="21" t="s">
+      <c r="D72" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="F72" s="21"/>
-      <c r="G72" s="21"/>
-      <c r="H72" s="21"/>
-      <c r="I72" s="15"/>
-      <c r="J72" s="15"/>
-      <c r="K72" s="15"/>
-      <c r="L72" s="15"/>
+      <c r="E72" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="F72" s="16"/>
+      <c r="G72" s="16"/>
+      <c r="H72" s="16"/>
+      <c r="I72" s="20"/>
+      <c r="J72" s="20"/>
+      <c r="K72" s="20"/>
+      <c r="L72" s="20"/>
     </row>
     <row r="73" spans="3:17">
-      <c r="C73" s="17">
+      <c r="C73" s="21">
         <v>3</v>
       </c>
-      <c r="D73" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="E73" s="21" t="s">
+      <c r="D73" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="F73" s="21"/>
-      <c r="G73" s="21"/>
-      <c r="H73" s="21"/>
-      <c r="I73" s="15"/>
-      <c r="J73" s="15"/>
-      <c r="K73" s="15"/>
-      <c r="L73" s="15"/>
+      <c r="E73" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="F73" s="16"/>
+      <c r="G73" s="16"/>
+      <c r="H73" s="16"/>
+      <c r="I73" s="20"/>
+      <c r="J73" s="20"/>
+      <c r="K73" s="20"/>
+      <c r="L73" s="20"/>
     </row>
     <row r="74" spans="3:17">
-      <c r="C74" s="17">
+      <c r="C74" s="21">
         <v>4</v>
       </c>
-      <c r="D74" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="E74" s="21" t="s">
+      <c r="D74" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="F74" s="21"/>
-      <c r="G74" s="21"/>
-      <c r="H74" s="21"/>
-      <c r="I74" s="15"/>
-      <c r="J74" s="15"/>
-      <c r="K74" s="15"/>
-      <c r="L74" s="15"/>
+      <c r="E74" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="F74" s="16"/>
+      <c r="G74" s="16"/>
+      <c r="H74" s="16"/>
+      <c r="I74" s="20"/>
+      <c r="J74" s="20"/>
+      <c r="K74" s="20"/>
+      <c r="L74" s="20"/>
     </row>
     <row r="75" spans="3:17">
-      <c r="C75" s="17">
+      <c r="C75" s="21">
         <v>5</v>
       </c>
-      <c r="D75" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="E75" s="21" t="s">
+      <c r="D75" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="F75" s="21"/>
-      <c r="G75" s="21"/>
-      <c r="H75" s="21"/>
-      <c r="I75" s="15"/>
-      <c r="J75" s="15"/>
-      <c r="K75" s="15"/>
-      <c r="L75" s="15"/>
+      <c r="E75" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="F75" s="16"/>
+      <c r="G75" s="16"/>
+      <c r="H75" s="16"/>
+      <c r="I75" s="20"/>
+      <c r="J75" s="20"/>
+      <c r="K75" s="20"/>
+      <c r="L75" s="20"/>
     </row>
     <row r="76" spans="3:17">
-      <c r="C76" s="17">
+      <c r="C76" s="21">
         <v>6</v>
       </c>
-      <c r="D76" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="E76" s="21" t="s">
+      <c r="D76" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="F76" s="21"/>
-      <c r="G76" s="21"/>
-      <c r="H76" s="21"/>
-      <c r="I76" s="15"/>
-      <c r="J76" s="15"/>
-      <c r="K76" s="15"/>
-      <c r="L76" s="15"/>
+      <c r="E76" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="F76" s="16"/>
+      <c r="G76" s="16"/>
+      <c r="H76" s="16"/>
+      <c r="I76" s="20"/>
+      <c r="J76" s="20"/>
+      <c r="K76" s="20"/>
+      <c r="L76" s="20"/>
     </row>
     <row r="77" spans="3:17">
-      <c r="C77" s="17">
+      <c r="C77" s="21">
         <v>7</v>
       </c>
-      <c r="D77" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="E77" s="21" t="s">
+      <c r="D77" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="F77" s="21"/>
-      <c r="G77" s="21"/>
-      <c r="H77" s="21"/>
-      <c r="I77" s="15"/>
-      <c r="J77" s="15"/>
-      <c r="K77" s="15"/>
-      <c r="L77" s="15"/>
+      <c r="E77" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="F77" s="16"/>
+      <c r="G77" s="16"/>
+      <c r="H77" s="16"/>
+      <c r="I77" s="20"/>
+      <c r="J77" s="20"/>
+      <c r="K77" s="20"/>
+      <c r="L77" s="20"/>
     </row>
     <row r="78" spans="3:17">
-      <c r="C78" s="17">
+      <c r="C78" s="21">
         <v>8</v>
       </c>
-      <c r="D78" s="16" t="s">
+      <c r="D78" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="E78" s="21" t="s">
+      <c r="E78" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="F78" s="21"/>
-      <c r="G78" s="21"/>
-      <c r="H78" s="21"/>
-      <c r="I78" s="15"/>
-      <c r="J78" s="15"/>
-      <c r="K78" s="15"/>
-      <c r="L78" s="15"/>
+      <c r="F78" s="16"/>
+      <c r="G78" s="16"/>
+      <c r="H78" s="16"/>
+      <c r="I78" s="20"/>
+      <c r="J78" s="20"/>
+      <c r="K78" s="20"/>
+      <c r="L78" s="20"/>
     </row>
     <row r="79" spans="3:17">
-      <c r="C79" s="17">
+      <c r="C79" s="21">
         <v>9</v>
       </c>
-      <c r="D79" s="16" t="s">
+      <c r="D79" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="E79" s="21" t="s">
+      <c r="E79" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F79" s="21"/>
-      <c r="G79" s="21"/>
-      <c r="H79" s="21"/>
-      <c r="I79" s="15"/>
-      <c r="J79" s="15"/>
-      <c r="K79" s="15"/>
-      <c r="L79" s="15"/>
+      <c r="F79" s="16"/>
+      <c r="G79" s="16"/>
+      <c r="H79" s="16"/>
+      <c r="I79" s="20"/>
+      <c r="J79" s="20"/>
+      <c r="K79" s="20"/>
+      <c r="L79" s="20"/>
     </row>
     <row r="80" spans="3:17">
-      <c r="C80" s="17">
+      <c r="C80" s="21">
         <v>10</v>
       </c>
-      <c r="D80" s="16" t="s">
+      <c r="D80" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="E80" s="21" t="s">
+      <c r="E80" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="F80" s="21"/>
-      <c r="G80" s="21"/>
-      <c r="H80" s="21"/>
-      <c r="I80" s="15"/>
-      <c r="J80" s="15"/>
-      <c r="K80" s="15"/>
-      <c r="L80" s="15"/>
-    </row>
-    <row r="81" spans="3:12">
-      <c r="C81" s="17">
+      <c r="F80" s="16"/>
+      <c r="G80" s="16"/>
+      <c r="H80" s="16"/>
+      <c r="I80" s="20"/>
+      <c r="J80" s="20"/>
+      <c r="K80" s="20"/>
+      <c r="L80" s="20"/>
+    </row>
+    <row r="81" spans="3:13">
+      <c r="C81" s="21">
         <v>11</v>
       </c>
-      <c r="D81" s="16" t="s">
+      <c r="D81" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="E81" s="21" t="s">
+      <c r="E81" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="F81" s="21"/>
-      <c r="G81" s="21"/>
-      <c r="H81" s="21"/>
-      <c r="I81" s="15"/>
-      <c r="J81" s="15"/>
-      <c r="K81" s="15"/>
-      <c r="L81" s="15"/>
-    </row>
-    <row r="82" spans="3:12">
-      <c r="C82" s="14"/>
-      <c r="D82" s="13"/>
-    </row>
-    <row r="83" spans="3:12">
-      <c r="C83" s="14"/>
-      <c r="D83" s="13"/>
-    </row>
-    <row r="84" spans="3:12">
-      <c r="C84" s="14"/>
-      <c r="D84" s="13"/>
-    </row>
-    <row r="85" spans="3:12">
-      <c r="C85" s="14"/>
-      <c r="D85" s="13"/>
-    </row>
-    <row r="86" spans="3:12">
-      <c r="C86" s="14"/>
-      <c r="D86" s="13"/>
+      <c r="F81" s="16"/>
+      <c r="G81" s="16"/>
+      <c r="H81" s="16"/>
+      <c r="I81" s="20"/>
+      <c r="J81" s="20"/>
+      <c r="K81" s="20"/>
+      <c r="L81" s="20"/>
+      <c r="M81" s="20"/>
+    </row>
+    <row r="82" spans="3:13">
+      <c r="C82" s="23"/>
+      <c r="D82" s="24"/>
+    </row>
+    <row r="83" spans="3:13">
+      <c r="C83" s="23"/>
+      <c r="D83" s="24"/>
+    </row>
+    <row r="84" spans="3:13">
+      <c r="C84" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="D84" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="E84" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="F84" s="26"/>
+      <c r="G84" s="26"/>
+      <c r="H84" s="26"/>
+      <c r="I84" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="J84" s="26"/>
+      <c r="K84" s="26"/>
+    </row>
+    <row r="85" spans="3:13">
+      <c r="C85" s="21">
+        <v>1</v>
+      </c>
+      <c r="D85" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="E85" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="F85" s="16"/>
+      <c r="G85" s="16"/>
+      <c r="H85" s="16"/>
+      <c r="I85" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="J85" s="16"/>
+      <c r="K85" s="16"/>
+    </row>
+    <row r="86" spans="3:13">
+      <c r="C86" s="21">
+        <v>2</v>
+      </c>
+      <c r="D86" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="E86" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="F86" s="16"/>
+      <c r="G86" s="16"/>
+      <c r="H86" s="16"/>
+      <c r="I86" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="J86" s="16"/>
+      <c r="K86" s="16"/>
+    </row>
+    <row r="87" spans="3:13">
+      <c r="C87" s="22">
+        <v>3</v>
+      </c>
+      <c r="D87" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="E87" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="F87" s="16"/>
+      <c r="G87" s="16"/>
+      <c r="H87" s="16"/>
+      <c r="I87" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="J87" s="16"/>
+      <c r="K87" s="16"/>
+    </row>
+    <row r="88" spans="3:13">
+      <c r="C88" s="21">
+        <v>4</v>
+      </c>
+      <c r="D88" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="E88" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="F88" s="16"/>
+      <c r="G88" s="16"/>
+      <c r="H88" s="16"/>
+      <c r="I88" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="J88" s="16"/>
+      <c r="K88" s="16"/>
+    </row>
+    <row r="89" spans="3:13">
+      <c r="C89" s="21">
+        <v>5</v>
+      </c>
+      <c r="D89" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="E89" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="F89" s="16"/>
+      <c r="G89" s="16"/>
+      <c r="H89" s="16"/>
+      <c r="I89" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="J89" s="16"/>
+      <c r="K89" s="16"/>
+    </row>
+    <row r="90" spans="3:13">
+      <c r="C90" s="21">
+        <v>6</v>
+      </c>
+      <c r="D90" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="E90" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="F90" s="16"/>
+      <c r="G90" s="16"/>
+      <c r="H90" s="16"/>
+      <c r="I90" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="J90" s="16"/>
+      <c r="K90" s="16"/>
+    </row>
+    <row r="91" spans="3:13">
+      <c r="C91" s="21">
+        <v>7</v>
+      </c>
+      <c r="D91" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="E91" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="F91" s="16"/>
+      <c r="G91" s="16"/>
+      <c r="H91" s="16"/>
+      <c r="I91" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="J91" s="16"/>
+      <c r="K91" s="16"/>
+    </row>
+    <row r="92" spans="3:13">
+      <c r="C92" s="21">
+        <v>8</v>
+      </c>
+      <c r="D92" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="E92" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="F92" s="16"/>
+      <c r="G92" s="16"/>
+      <c r="H92" s="16"/>
+      <c r="I92" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="J92" s="16"/>
+      <c r="K92" s="16"/>
+    </row>
+    <row r="93" spans="3:13">
+      <c r="C93" s="22">
+        <v>9</v>
+      </c>
+      <c r="D93" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="E93" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="F93" s="16"/>
+      <c r="G93" s="16"/>
+      <c r="H93" s="16"/>
+      <c r="I93" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="J93" s="16"/>
+      <c r="K93" s="16"/>
+    </row>
+    <row r="94" spans="3:13">
+      <c r="C94" s="21">
+        <v>10</v>
+      </c>
+      <c r="D94" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="E94" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="F94" s="16"/>
+      <c r="G94" s="16"/>
+      <c r="H94" s="16"/>
+      <c r="I94" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="J94" s="16"/>
+      <c r="K94" s="16"/>
+    </row>
+    <row r="95" spans="3:13">
+      <c r="C95" s="21">
+        <v>11</v>
+      </c>
+      <c r="D95" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="E95" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="F95" s="16"/>
+      <c r="G95" s="16"/>
+      <c r="H95" s="16"/>
+      <c r="I95" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="J95" s="16"/>
+      <c r="K95" s="16"/>
+    </row>
+    <row r="96" spans="3:13">
+      <c r="C96" s="21">
+        <v>12</v>
+      </c>
+      <c r="D96" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="E96" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="F96" s="16"/>
+      <c r="G96" s="16"/>
+      <c r="H96" s="16"/>
+      <c r="I96" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="J96" s="16"/>
+      <c r="K96" s="16"/>
+    </row>
+    <row r="97" spans="3:11">
+      <c r="C97" s="21">
+        <v>13</v>
+      </c>
+      <c r="D97" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="E97" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="F97" s="16"/>
+      <c r="G97" s="16"/>
+      <c r="H97" s="16"/>
+      <c r="I97" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="J97" s="16"/>
+      <c r="K97" s="16"/>
+    </row>
+    <row r="98" spans="3:11">
+      <c r="C98" s="21">
+        <v>14</v>
+      </c>
+      <c r="D98" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="E98" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="F98" s="16"/>
+      <c r="G98" s="16"/>
+      <c r="H98" s="16"/>
+      <c r="I98" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="J98" s="16"/>
+      <c r="K98" s="16"/>
+    </row>
+    <row r="99" spans="3:11">
+      <c r="C99" s="22">
+        <v>15</v>
+      </c>
+      <c r="D99" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="E99" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="F99" s="16"/>
+      <c r="G99" s="16"/>
+      <c r="H99" s="16"/>
+      <c r="I99" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="J99" s="16"/>
+      <c r="K99" s="16"/>
+    </row>
+    <row r="100" spans="3:11">
+      <c r="C100" s="21">
+        <v>16</v>
+      </c>
+      <c r="D100" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="E100" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="F100" s="16"/>
+      <c r="G100" s="16"/>
+      <c r="H100" s="16"/>
+      <c r="I100" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="J100" s="16"/>
+      <c r="K100" s="16"/>
+    </row>
+    <row r="101" spans="3:11">
+      <c r="C101" s="21">
+        <v>17</v>
+      </c>
+      <c r="D101" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="E101" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="F101" s="16"/>
+      <c r="G101" s="16"/>
+      <c r="H101" s="16"/>
+      <c r="I101" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="J101" s="16"/>
+      <c r="K101" s="16"/>
+    </row>
+    <row r="102" spans="3:11">
+      <c r="C102" s="21">
+        <v>18</v>
+      </c>
+      <c r="D102" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="E102" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="F102" s="16"/>
+      <c r="G102" s="16"/>
+      <c r="H102" s="16"/>
+      <c r="I102" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="J102" s="16"/>
+      <c r="K102" s="16"/>
+    </row>
+    <row r="103" spans="3:11">
+      <c r="C103" s="21">
+        <v>19</v>
+      </c>
+      <c r="D103" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="E103" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="F103" s="16"/>
+      <c r="G103" s="16"/>
+      <c r="H103" s="16"/>
+      <c r="I103" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="J103" s="16"/>
+      <c r="K103" s="16"/>
+    </row>
+    <row r="104" spans="3:11">
+      <c r="C104" s="21">
+        <v>20</v>
+      </c>
+      <c r="D104" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="E104" s="16" t="s">
+        <v>162</v>
+      </c>
+      <c r="F104" s="16"/>
+      <c r="G104" s="16"/>
+      <c r="H104" s="16"/>
+      <c r="I104" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="J104" s="16"/>
+      <c r="K104" s="16"/>
+    </row>
+    <row r="105" spans="3:11">
+      <c r="C105" s="22">
+        <v>21</v>
+      </c>
+      <c r="D105" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="E105" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="F105" s="16"/>
+      <c r="G105" s="16"/>
+      <c r="H105" s="16"/>
+      <c r="I105" s="16" t="s">
+        <v>166</v>
+      </c>
+      <c r="J105" s="16"/>
+      <c r="K105" s="16"/>
+    </row>
+    <row r="106" spans="3:11">
+      <c r="C106" s="21">
+        <v>22</v>
+      </c>
+      <c r="D106" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="E106" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="F106" s="16"/>
+      <c r="G106" s="16"/>
+      <c r="H106" s="16"/>
+      <c r="I106" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="J106" s="16"/>
+      <c r="K106" s="16"/>
+    </row>
+    <row r="107" spans="3:11">
+      <c r="C107" s="21">
+        <v>23</v>
+      </c>
+      <c r="D107" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="E107" s="16" t="s">
+        <v>171</v>
+      </c>
+      <c r="F107" s="16"/>
+      <c r="G107" s="16"/>
+      <c r="H107" s="16"/>
+      <c r="I107" s="16" t="s">
+        <v>172</v>
+      </c>
+      <c r="J107" s="16"/>
+      <c r="K107" s="16"/>
+    </row>
+    <row r="108" spans="3:11">
+      <c r="C108" s="21">
+        <v>24</v>
+      </c>
+      <c r="D108" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="E108" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="F108" s="16"/>
+      <c r="G108" s="16"/>
+      <c r="H108" s="16"/>
+      <c r="I108" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="J108" s="16"/>
+      <c r="K108" s="16"/>
+    </row>
+    <row r="109" spans="3:11">
+      <c r="C109" s="21">
+        <v>25</v>
+      </c>
+      <c r="D109" s="22" t="s">
+        <v>176</v>
+      </c>
+      <c r="E109" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="F109" s="16"/>
+      <c r="G109" s="16"/>
+      <c r="H109" s="16"/>
+      <c r="I109" s="16" t="s">
+        <v>177</v>
+      </c>
+      <c r="J109" s="16"/>
+      <c r="K109" s="16"/>
+    </row>
+    <row r="110" spans="3:11">
+      <c r="C110" s="21">
+        <v>26</v>
+      </c>
+      <c r="D110" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="E110" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="F110" s="16"/>
+      <c r="G110" s="16"/>
+      <c r="H110" s="16"/>
+      <c r="I110" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="J110" s="16"/>
+      <c r="K110" s="16"/>
+    </row>
+    <row r="111" spans="3:11">
+      <c r="C111" s="22">
+        <v>27</v>
+      </c>
+      <c r="D111" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="E111" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="F111" s="16"/>
+      <c r="G111" s="16"/>
+      <c r="H111" s="16"/>
+      <c r="I111" s="16" t="s">
+        <v>182</v>
+      </c>
+      <c r="J111" s="16"/>
+      <c r="K111" s="16"/>
+    </row>
+    <row r="112" spans="3:11">
+      <c r="C112" s="21">
+        <v>28</v>
+      </c>
+      <c r="D112" s="22" t="s">
+        <v>183</v>
+      </c>
+      <c r="E112" s="16" t="s">
+        <v>184</v>
+      </c>
+      <c r="F112" s="16"/>
+      <c r="G112" s="16"/>
+      <c r="H112" s="16"/>
+      <c r="I112" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="J112" s="16"/>
+      <c r="K112" s="16"/>
+    </row>
+    <row r="113" spans="3:11">
+      <c r="C113" s="21">
+        <v>29</v>
+      </c>
+      <c r="D113" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="E113" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="F113" s="16"/>
+      <c r="G113" s="16"/>
+      <c r="H113" s="16"/>
+      <c r="I113" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="J113" s="16"/>
+      <c r="K113" s="16"/>
+    </row>
+    <row r="114" spans="3:11">
+      <c r="E114" s="25"/>
+      <c r="F114" s="25"/>
+      <c r="G114" s="25"/>
+      <c r="H114" s="25"/>
+    </row>
+    <row r="115" spans="3:11">
+      <c r="E115" s="25"/>
+      <c r="F115" s="25"/>
+      <c r="G115" s="25"/>
+      <c r="H115" s="25"/>
+    </row>
+    <row r="116" spans="3:11">
+      <c r="E116" s="25"/>
+      <c r="F116" s="25"/>
+      <c r="G116" s="25"/>
+      <c r="H116" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="77">
+    <mergeCell ref="E113:H113"/>
+    <mergeCell ref="I113:K113"/>
+    <mergeCell ref="E114:H114"/>
+    <mergeCell ref="E115:H115"/>
+    <mergeCell ref="E116:H116"/>
+    <mergeCell ref="E110:H110"/>
+    <mergeCell ref="I110:K110"/>
+    <mergeCell ref="E111:H111"/>
+    <mergeCell ref="I111:K111"/>
+    <mergeCell ref="E112:H112"/>
+    <mergeCell ref="I112:K112"/>
+    <mergeCell ref="E107:H107"/>
+    <mergeCell ref="I107:K107"/>
+    <mergeCell ref="E108:H108"/>
+    <mergeCell ref="I108:K108"/>
+    <mergeCell ref="E109:H109"/>
+    <mergeCell ref="I109:K109"/>
+    <mergeCell ref="E104:H104"/>
+    <mergeCell ref="I104:K104"/>
+    <mergeCell ref="E105:H105"/>
+    <mergeCell ref="I105:K105"/>
+    <mergeCell ref="E106:H106"/>
+    <mergeCell ref="I106:K106"/>
+    <mergeCell ref="E101:H101"/>
+    <mergeCell ref="I101:K101"/>
+    <mergeCell ref="E102:H102"/>
+    <mergeCell ref="I102:K102"/>
+    <mergeCell ref="E103:H103"/>
+    <mergeCell ref="I103:K103"/>
+    <mergeCell ref="E98:H98"/>
+    <mergeCell ref="I98:K98"/>
+    <mergeCell ref="E99:H99"/>
+    <mergeCell ref="I99:K99"/>
+    <mergeCell ref="E100:H100"/>
+    <mergeCell ref="I100:K100"/>
+    <mergeCell ref="E95:H95"/>
+    <mergeCell ref="I95:K95"/>
+    <mergeCell ref="E96:H96"/>
+    <mergeCell ref="I96:K96"/>
+    <mergeCell ref="E97:H97"/>
+    <mergeCell ref="I97:K97"/>
+    <mergeCell ref="E92:H92"/>
+    <mergeCell ref="I92:K92"/>
+    <mergeCell ref="E93:H93"/>
+    <mergeCell ref="I93:K93"/>
+    <mergeCell ref="E94:H94"/>
+    <mergeCell ref="I94:K94"/>
+    <mergeCell ref="E89:H89"/>
+    <mergeCell ref="I89:K89"/>
+    <mergeCell ref="E90:H90"/>
+    <mergeCell ref="I90:K90"/>
+    <mergeCell ref="E91:H91"/>
+    <mergeCell ref="I91:K91"/>
+    <mergeCell ref="E86:H86"/>
+    <mergeCell ref="I86:K86"/>
+    <mergeCell ref="E87:H87"/>
+    <mergeCell ref="I87:K87"/>
+    <mergeCell ref="E88:H88"/>
+    <mergeCell ref="I88:K88"/>
     <mergeCell ref="E80:H80"/>
     <mergeCell ref="E81:H81"/>
+    <mergeCell ref="E84:H84"/>
+    <mergeCell ref="I84:K84"/>
+    <mergeCell ref="E85:H85"/>
+    <mergeCell ref="I85:K85"/>
     <mergeCell ref="E74:H74"/>
     <mergeCell ref="E75:H75"/>
     <mergeCell ref="E76:H76"/>
     <mergeCell ref="E77:H77"/>
     <mergeCell ref="E78:H78"/>
     <mergeCell ref="E79:H79"/>
-    <mergeCell ref="E73:H73"/>
     <mergeCell ref="N65:Q65"/>
-    <mergeCell ref="C69:L69"/>
+    <mergeCell ref="C69:H69"/>
     <mergeCell ref="E70:H70"/>
     <mergeCell ref="E71:H71"/>
     <mergeCell ref="E72:H72"/>
+    <mergeCell ref="E73:H73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: CAN/LIN gui updated
</commit_message>
<xml_diff>
--- a/SmartBU/How_To_Debugg.xlsx
+++ b/SmartBU/How_To_Debugg.xlsx
@@ -9,24 +9,26 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9070" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9070" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Revision_1.0" sheetId="1" r:id="rId1"/>
     <sheet name="Revision_1.1" sheetId="2" r:id="rId2"/>
-    <sheet name="Connection " sheetId="4" r:id="rId3"/>
+    <sheet name="Auto_Install" sheetId="5" r:id="rId3"/>
+    <sheet name="KIKUSUI PWR401L SETUP STEPS " sheetId="6" r:id="rId4"/>
+    <sheet name="Connection " sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="MXAj33uNO1zcz6WY6d6qq3mLHNVLbJybT5QnkKJAJAQ="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="MXAj33uNO1zcz6WY6d6qq3mLHNVLbJybT5QnkKJAJAQ="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="225">
   <si>
     <t>Project Setup Using Trace32</t>
   </si>
@@ -693,64 +695,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">2. Open the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Testbench_gui/ManualTest</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> project directory.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Open the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Testbench_gui</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> project directory.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">2. Run </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>run_automation_gui.</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">3. Click </t>
     </r>
     <r>
@@ -773,9 +717,6 @@
     </r>
   </si>
   <si>
-    <t>4. Select the variant according to your connected hardware.</t>
-  </si>
-  <si>
     <t>Capa Singal Dip Switch 100pF</t>
   </si>
   <si>
@@ -1038,13 +979,206 @@
   </si>
   <si>
     <t>PIN 28</t>
+  </si>
+  <si>
+    <t>...\Testbench_gui_Rev1.1\Tools\Auto_Install</t>
+  </si>
+  <si>
+    <t>Brouse the path</t>
+  </si>
+  <si>
+    <t>Double click on Run_Auto_Install.bat</t>
+  </si>
+  <si>
+    <t>Wait for installation completion</t>
+  </si>
+  <si>
+    <t>Check similar with screen shot</t>
+  </si>
+  <si>
+    <t>--------------------------------------------------------------------------------</t>
+  </si>
+  <si>
+    <t>KIKUSUI PWR401L SETUP STEPS (for Japan colleague)</t>
+  </si>
+  <si>
+    <t>STEP 1 - Install instrument driver/runtime (Windows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Install NI-VISA Runtime (recommended):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    https://www.ni.com/en/support/downloads/drivers/download.ni-visa.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Notes:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    - This provides visa32/visa64 backend required by PyVISA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    - Reboot after install if prompted.</t>
+  </si>
+  <si>
+    <t>STEP 2 - Connect KIKUSUI PSU and verify Device Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Connect KIKUSUI PWR401L over USB (USBTMC) or configured VISA interface.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Confirm it appears under VISA/USB test instrument category without warning icon.</t>
+  </si>
+  <si>
+    <t>STEP 3 - Install Python libraries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  From project root run:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    pip install -r requirements.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Added libraries:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    - pyvisa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    - pyvisa-py (fallback backend)</t>
+  </si>
+  <si>
+    <t>STEP 4 - Verify VISA sees the PSU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Run:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    python -c "import pyvisa; rm=pyvisa.ResourceManager(); print(rm.list_resources())"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Expected: at least one USB/TCPIP VISA resource for the KIKUSUI unit.</t>
+  </si>
+  <si>
+    <t>STEP 5 - Select PSU type before running automation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  PowerShell (same terminal where app is launched):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    $env:PSU_TYPE = "kikusui"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Optional explicit resource (if auto-detect picks wrong instrument):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    $env:KIKUSUI_PSU_RESOURCE = "USB0::....::INSTR"</t>
+  </si>
+  <si>
+    <t>STEP 6 - Run GUI automation normally</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  The app will now use KIKUSUI backend for ON/OFF and voltage/current SCPI commands.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2. Run </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>AutomationTest.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Open the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Testbench_gui_Rev1.1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> project directory.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2. Open the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Testbench_gui_Rev1.1/ManualTest</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> project directory.</t>
+    </r>
+  </si>
+  <si>
+    <t>pip install pyserial</t>
+  </si>
+  <si>
+    <t>pip install pandas</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/1ImQWcyVE9dQLkQHOCaHPdNoRTm6heKEl</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">Download the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Testbench_gui_Rev1.1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> from the following Google Drive link:</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1160,6 +1294,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1206,13 +1347,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1274,20 +1416,23 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="5">
+    <cellStyle name="Hyperlink" xfId="4" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2"/>
     <cellStyle name="Normal 3" xfId="3"/>
@@ -1967,7 +2112,7 @@
     <xdr:from>
       <xdr:col>12</xdr:col>
       <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>161</xdr:row>
+      <xdr:row>164</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1743075" cy="723900"/>
@@ -2025,7 +2170,7 @@
     <xdr:from>
       <xdr:col>12</xdr:col>
       <xdr:colOff>323850</xdr:colOff>
-      <xdr:row>185</xdr:row>
+      <xdr:row>188</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1743075" cy="723900"/>
@@ -2083,7 +2228,7 @@
     <xdr:from>
       <xdr:col>12</xdr:col>
       <xdr:colOff>390525</xdr:colOff>
-      <xdr:row>211</xdr:row>
+      <xdr:row>214</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1743075" cy="723900"/>
@@ -2205,7 +2350,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>99</xdr:row>
+      <xdr:row>102</xdr:row>
       <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6343650" cy="3409950"/>
@@ -2269,7 +2414,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>260</xdr:row>
+      <xdr:row>263</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6296025" cy="4171950"/>
@@ -2301,7 +2446,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>288</xdr:row>
+      <xdr:row>291</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6296025" cy="4619625"/>
@@ -2333,39 +2478,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>126</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6457950" cy="3333750"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="image7.png"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="609600" y="22802850"/>
-          <a:ext cx="6457950" cy="3333750"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>177</xdr:row>
+      <xdr:row>180</xdr:row>
       <xdr:rowOff>142875</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6400800" cy="3829050"/>
@@ -2375,7 +2488,7 @@
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2397,7 +2510,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>153</xdr:row>
+      <xdr:row>156</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6362700" cy="3810000"/>
@@ -2407,7 +2520,7 @@
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2429,7 +2542,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>203</xdr:row>
+      <xdr:row>206</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6467475" cy="3829050"/>
@@ -2439,7 +2552,7 @@
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2461,7 +2574,7 @@
     <xdr:from>
       <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>153</xdr:row>
+      <xdr:row>156</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6267450" cy="3714750"/>
@@ -2471,7 +2584,7 @@
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2493,7 +2606,7 @@
     <xdr:from>
       <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>178</xdr:row>
+      <xdr:row>181</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6238875" cy="3676650"/>
@@ -2503,7 +2616,7 @@
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2525,7 +2638,7 @@
     <xdr:from>
       <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>203</xdr:row>
+      <xdr:row>206</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6296025" cy="3914775"/>
@@ -2535,7 +2648,7 @@
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2557,7 +2670,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>571500</xdr:colOff>
-      <xdr:row>316</xdr:row>
+      <xdr:row>319</xdr:row>
       <xdr:rowOff>190500</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6296025" cy="4191000"/>
@@ -2567,7 +2680,7 @@
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2589,7 +2702,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>581025</xdr:colOff>
-      <xdr:row>348</xdr:row>
+      <xdr:row>351</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6591300" cy="4429125"/>
@@ -2599,7 +2712,7 @@
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2621,7 +2734,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>379</xdr:row>
+      <xdr:row>382</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6362700" cy="4848225"/>
@@ -2631,7 +2744,7 @@
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2653,13 +2766,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>232</xdr:row>
+      <xdr:row>235</xdr:row>
       <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>428371</xdr:colOff>
-      <xdr:row>251</xdr:row>
+      <xdr:row>254</xdr:row>
       <xdr:rowOff>53164</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2670,7 +2783,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2689,20 +2802,58 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>51662</xdr:colOff>
-      <xdr:row>413</xdr:row>
-      <xdr:rowOff>116237</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>546654</xdr:colOff>
+      <xdr:row>428</xdr:row>
+      <xdr:rowOff>60740</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>32097</xdr:colOff>
-      <xdr:row>433</xdr:row>
-      <xdr:rowOff>25831</xdr:rowOff>
+      <xdr:colOff>42889</xdr:colOff>
+      <xdr:row>439</xdr:row>
+      <xdr:rowOff>71784</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="23" name="Picture 22"/>
+        <xdr:cNvPr id="9" name="Picture 8"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="546654" y="77591479"/>
+          <a:ext cx="6917452" cy="1954696"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>16565</xdr:colOff>
+      <xdr:row>416</xdr:row>
+      <xdr:rowOff>49696</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>353147</xdr:colOff>
+      <xdr:row>425</xdr:row>
+      <xdr:rowOff>110435</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Picture 23"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -2715,8 +2866,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="658679" y="75450915"/>
-          <a:ext cx="6657621" cy="3525865"/>
+          <a:off x="635000" y="73516435"/>
+          <a:ext cx="6520930" cy="1651000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2729,18 +2880,18 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>437</xdr:row>
+      <xdr:row>129</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>45719</xdr:colOff>
-      <xdr:row>457</xdr:row>
-      <xdr:rowOff>4563</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>261996</xdr:colOff>
+      <xdr:row>147</xdr:row>
+      <xdr:rowOff>33130</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="25" name="Picture 24"/>
+        <xdr:cNvPr id="27" name="Picture 26"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -2753,46 +2904,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="609600" y="80573880"/>
-          <a:ext cx="6751319" cy="3652465"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>460</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>45180</xdr:colOff>
-      <xdr:row>479</xdr:row>
-      <xdr:rowOff>106681</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="26" name="Picture 25"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="609600" y="84780120"/>
-          <a:ext cx="6750780" cy="3581400"/>
+          <a:off x="618435" y="23014609"/>
+          <a:ext cx="8920083" cy="3213651"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2805,6 +2918,49 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>368943</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>166201</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2921000" y="1117600"/>
+          <a:ext cx="4610743" cy="7887801"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -5631,7 +5787,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:Q1079"/>
+  <dimension ref="B1:Q1040"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="27" width="8.81640625" customWidth="1"/>
@@ -5694,7 +5850,7 @@
     </row>
     <row r="18" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="19" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="29" t="s">
         <v>9</v>
       </c>
     </row>
@@ -5823,38 +5979,50 @@
     </row>
     <row r="93" spans="2:2" ht="14.25" customHeight="1">
       <c r="B93" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="94" spans="2:2" ht="14.25" customHeight="1">
       <c r="B94" s="5" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="95" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B95" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="96" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B96" s="5" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="97" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B97" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="95" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B95" s="11" t="s">
+    <row r="98" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B98" s="11" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="96" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B96" s="11" t="s">
+    <row r="99" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B99" s="11" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="97" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B97" s="11" t="s">
+    <row r="100" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B100" s="11" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="98" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="99" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B99" s="1" t="s">
+    <row r="101" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="102" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B102" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="100" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="101" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="102" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="103" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="104" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="105" spans="2:2" ht="14.25" customHeight="1"/>
@@ -5873,26 +6041,26 @@
     <row r="118" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="119" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="120" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="121" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B121" s="2" t="s">
+    <row r="121" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="122" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="123" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="124" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B124" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="122" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="123" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B123" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="124" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="125" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B125" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="126" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="125" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="126" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B126" s="30" t="s">
+        <v>224</v>
+      </c>
+    </row>
     <row r="127" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="128" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="128" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B128" s="29" t="s">
+        <v>223</v>
+      </c>
+    </row>
     <row r="129" ht="14.25" customHeight="1"/>
     <row r="130" ht="14.25" customHeight="1"/>
     <row r="131" ht="14.25" customHeight="1"/>
@@ -5911,79 +6079,79 @@
     <row r="144" ht="14.25" customHeight="1"/>
     <row r="145" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="146" spans="2:17" ht="14.25" customHeight="1"/>
-    <row r="147" spans="2:17" ht="14.25" customHeight="1">
-      <c r="B147" s="2" t="s">
+    <row r="147" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="148" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="149" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="150" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B150" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="148" spans="2:17" ht="14.25" customHeight="1">
-      <c r="B148" s="8"/>
-    </row>
-    <row r="149" spans="2:17" ht="14.25" customHeight="1">
-      <c r="B149" s="8" t="s">
+    <row r="151" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B151" s="8"/>
+    </row>
+    <row r="152" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B152" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="150" spans="2:17" ht="14.25" customHeight="1">
-      <c r="B150" s="8"/>
-    </row>
-    <row r="151" spans="2:17" ht="14.25" customHeight="1">
-      <c r="B151" s="7" t="s">
+    <row r="153" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B153" s="8"/>
+    </row>
+    <row r="154" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B154" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q151" s="1" t="s">
+      <c r="Q154" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="152" spans="2:17" ht="14.25" customHeight="1">
-      <c r="B152" s="7" t="s">
+    <row r="155" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B155" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="Q152" s="7" t="s">
+      <c r="Q155" s="7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="153" spans="2:17" ht="14.25" customHeight="1"/>
-    <row r="154" spans="2:17" ht="14.25" customHeight="1"/>
-    <row r="155" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="156" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="157" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="158" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="159" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="160" spans="2:17" ht="14.25" customHeight="1"/>
-    <row r="161" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="162" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="163" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="164" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="165" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="166" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="167" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="168" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="169" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="170" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="171" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="172" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="173" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="174" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="175" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B175" s="8"/>
-    </row>
-    <row r="176" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B176" s="7" t="s">
+    <row r="161" ht="14.25" customHeight="1"/>
+    <row r="162" ht="14.25" customHeight="1"/>
+    <row r="163" ht="14.25" customHeight="1"/>
+    <row r="164" ht="14.25" customHeight="1"/>
+    <row r="165" ht="14.25" customHeight="1"/>
+    <row r="166" ht="14.25" customHeight="1"/>
+    <row r="167" ht="14.25" customHeight="1"/>
+    <row r="168" ht="14.25" customHeight="1"/>
+    <row r="169" ht="14.25" customHeight="1"/>
+    <row r="170" ht="14.25" customHeight="1"/>
+    <row r="171" ht="14.25" customHeight="1"/>
+    <row r="172" ht="14.25" customHeight="1"/>
+    <row r="173" ht="14.25" customHeight="1"/>
+    <row r="174" ht="14.25" customHeight="1"/>
+    <row r="175" ht="14.25" customHeight="1"/>
+    <row r="176" ht="14.25" customHeight="1"/>
+    <row r="177" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="178" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B178" s="8"/>
+    </row>
+    <row r="179" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B179" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="177" spans="2:17" ht="14.25" customHeight="1">
-      <c r="B177" s="7" t="s">
+    <row r="180" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B180" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="Q177" s="7" t="s">
+      <c r="Q180" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="178" spans="2:17" ht="14.25" customHeight="1"/>
-    <row r="179" spans="2:17" ht="14.25" customHeight="1"/>
-    <row r="180" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="181" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="182" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="183" spans="2:17" ht="14.25" customHeight="1"/>
@@ -6004,22 +6172,22 @@
     <row r="198" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="199" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="200" spans="2:17" ht="14.25" customHeight="1"/>
-    <row r="201" spans="2:17" ht="14.25" customHeight="1">
-      <c r="B201" s="7" t="s">
+    <row r="201" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="202" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="203" spans="2:17" ht="14.25" customHeight="1"/>
+    <row r="204" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B204" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="202" spans="2:17" ht="14.25" customHeight="1">
-      <c r="B202" s="7" t="s">
+    <row r="205" spans="2:17" ht="14.25" customHeight="1">
+      <c r="B205" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="Q202" s="7" t="s">
+      <c r="Q205" s="7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="203" spans="2:17" ht="14.25" customHeight="1"/>
-    <row r="204" spans="2:17" ht="14.25" customHeight="1"/>
-    <row r="205" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="206" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="207" spans="2:17" ht="14.25" customHeight="1"/>
     <row r="208" spans="2:17" ht="14.25" customHeight="1"/>
@@ -6041,32 +6209,32 @@
     <row r="224" ht="14.25" customHeight="1"/>
     <row r="225" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="226" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="227" spans="2:2" ht="22.25" customHeight="1">
-      <c r="B227" s="2" t="s">
+    <row r="227" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="228" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="229" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="230" spans="2:2" ht="22.25" customHeight="1">
+      <c r="B230" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="228" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B228" s="8"/>
-    </row>
-    <row r="229" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B229" s="8" t="s">
+    <row r="231" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B231" s="8"/>
+    </row>
+    <row r="232" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B232" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="230" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B230" s="8" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="231" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B231" s="8" t="s">
+    <row r="233" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B233" s="8" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="234" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B234" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="232" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="233" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="234" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="235" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="236" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="237" spans="2:2" ht="14.25" customHeight="1"/>
@@ -6085,43 +6253,37 @@
     <row r="250" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="251" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="252" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="253" spans="2:2" ht="18.5" customHeight="1">
-      <c r="B253" s="2" t="s">
+    <row r="253" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="254" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="255" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="256" spans="2:2" ht="18.5" customHeight="1">
+      <c r="B256" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="254" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="255" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B255" s="1" t="s">
+    <row r="257" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="258" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B258" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="256" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B256" s="8"/>
-    </row>
-    <row r="257" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B257" s="9" t="s">
+    <row r="259" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B259" s="8"/>
+    </row>
+    <row r="260" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B260" s="9" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="258" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B258" s="8" t="s">
+    <row r="261" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B261" s="8" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="259" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B259" s="8" t="s">
+    <row r="262" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B262" s="8" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="260" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B260" s="8"/>
-    </row>
-    <row r="261" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B261" s="8"/>
-    </row>
-    <row r="262" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B262" s="8"/>
     </row>
     <row r="263" spans="2:2" ht="14.25" customHeight="1">
       <c r="B263" s="8"/>
@@ -6193,23 +6355,23 @@
       <c r="B285" s="8"/>
     </row>
     <row r="286" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B286" s="9" t="s">
-        <v>49</v>
-      </c>
+      <c r="B286" s="8"/>
     </row>
     <row r="287" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B287" s="8" t="s">
-        <v>50</v>
-      </c>
+      <c r="B287" s="8"/>
     </row>
     <row r="288" spans="2:2" ht="14.25" customHeight="1">
       <c r="B288" s="8"/>
     </row>
     <row r="289" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B289" s="8"/>
+      <c r="B289" s="9" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="290" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B290" s="8"/>
+      <c r="B290" s="8" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="291" spans="2:2" ht="14.25" customHeight="1">
       <c r="B291" s="8"/>
@@ -6287,18 +6449,24 @@
       <c r="B315" s="8"/>
     </row>
     <row r="316" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B316" s="9" t="s">
+      <c r="B316" s="8"/>
+    </row>
+    <row r="317" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B317" s="8"/>
+    </row>
+    <row r="318" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B318" s="8"/>
+    </row>
+    <row r="319" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B319" s="9" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="317" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B317" s="8" t="s">
+    <row r="320" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B320" s="8" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="318" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="319" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="320" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="321" ht="14.25" customHeight="1"/>
     <row r="322" ht="14.25" customHeight="1"/>
     <row r="323" ht="14.25" customHeight="1"/>
@@ -6322,32 +6490,32 @@
     <row r="341" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="342" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="343" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="344" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B344" s="2" t="s">
+    <row r="344" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="345" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="346" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="347" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B347" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="345" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B345" s="8"/>
-    </row>
-    <row r="346" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B346" s="8" t="s">
+    <row r="348" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B348" s="8"/>
+    </row>
+    <row r="349" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B349" s="8" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="347" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B347" s="8" t="s">
+    <row r="350" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B350" s="8" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="348" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B348" s="8" t="s">
+    <row r="351" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B351" s="8" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="349" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="350" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="351" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="352" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="353" ht="14.25" customHeight="1"/>
     <row r="354" ht="14.25" customHeight="1"/>
@@ -6370,36 +6538,36 @@
     <row r="371" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="372" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="373" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="374" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B374" s="1" t="s">
+    <row r="374" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="375" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="376" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="377" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B377" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="375" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="376" spans="2:2" ht="22.25" customHeight="1">
-      <c r="B376" s="2" t="s">
+    <row r="378" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="379" spans="2:2" ht="22.25" customHeight="1">
+      <c r="B379" s="2" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="377" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B377" s="8"/>
-    </row>
-    <row r="378" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B378" s="8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="379" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B379" s="8" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="380" spans="2:2" ht="14.25" customHeight="1">
       <c r="B380" s="8"/>
     </row>
-    <row r="381" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="382" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="383" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="381" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B381" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="382" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B382" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="383" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B383" s="8"/>
+    </row>
     <row r="384" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="385" ht="14.25" customHeight="1"/>
     <row r="386" ht="14.25" customHeight="1"/>
@@ -6426,81 +6594,95 @@
     <row r="407" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="408" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="409" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="410" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B410" s="12" t="s">
+    <row r="410" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="411" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="412" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="413" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B413" s="12" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="411" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="412" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B412" s="8" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="413" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B413" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
     <row r="414" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="415" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="416" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="417" ht="14.25" customHeight="1"/>
-    <row r="418" ht="14.25" customHeight="1"/>
-    <row r="419" ht="14.25" customHeight="1"/>
-    <row r="420" ht="14.25" customHeight="1"/>
-    <row r="421" ht="14.25" customHeight="1"/>
-    <row r="422" ht="14.25" customHeight="1"/>
-    <row r="423" ht="14.25" customHeight="1"/>
-    <row r="424" ht="14.25" customHeight="1"/>
-    <row r="425" ht="14.25" customHeight="1"/>
-    <row r="426" ht="14.25" customHeight="1"/>
-    <row r="427" ht="14.25" customHeight="1"/>
-    <row r="428" ht="14.25" customHeight="1"/>
-    <row r="429" ht="14.25" customHeight="1"/>
-    <row r="430" ht="14.25" customHeight="1"/>
-    <row r="431" ht="14.25" customHeight="1"/>
-    <row r="432" ht="14.25" customHeight="1"/>
+    <row r="415" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B415" s="8" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="416" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B416" s="8" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="417" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="418" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="419" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="420" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="421" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="422" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="423" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="424" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="425" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="426" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="427" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="428" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B428" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="429" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="430" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="431" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="432" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="433" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="434" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="435" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="436" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B436" s="13" t="s">
-        <v>99</v>
-      </c>
-    </row>
+    <row r="436" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="437" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="438" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="439" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="440" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="441" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="442" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="443" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="444" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="445" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="446" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="447" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="443" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B443" s="12" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="444" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B444" s="8"/>
+    </row>
+    <row r="445" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B445" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="446" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B446" s="8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="447" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B447" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
     <row r="448" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="449" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="450" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="451" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="452" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="453" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="454" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="455" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="456" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="457" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="458" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="459" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B459" s="13" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="460" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="461" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="462" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="463" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="464" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="449" ht="14.25" customHeight="1"/>
+    <row r="450" ht="14.25" customHeight="1"/>
+    <row r="451" ht="14.25" customHeight="1"/>
+    <row r="452" ht="14.25" customHeight="1"/>
+    <row r="453" ht="14.25" customHeight="1"/>
+    <row r="454" ht="14.25" customHeight="1"/>
+    <row r="455" ht="14.25" customHeight="1"/>
+    <row r="456" ht="14.25" customHeight="1"/>
+    <row r="457" ht="14.25" customHeight="1"/>
+    <row r="458" ht="14.25" customHeight="1"/>
+    <row r="459" ht="14.25" customHeight="1"/>
+    <row r="460" ht="14.25" customHeight="1"/>
+    <row r="461" ht="14.25" customHeight="1"/>
+    <row r="462" ht="14.25" customHeight="1"/>
+    <row r="463" ht="14.25" customHeight="1"/>
+    <row r="464" ht="14.25" customHeight="1"/>
     <row r="465" ht="14.25" customHeight="1"/>
     <row r="466" ht="14.25" customHeight="1"/>
     <row r="467" ht="14.25" customHeight="1"/>
@@ -6517,40 +6699,22 @@
     <row r="478" ht="14.25" customHeight="1"/>
     <row r="479" ht="14.25" customHeight="1"/>
     <row r="480" ht="14.25" customHeight="1"/>
-    <row r="481" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="482" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B482" s="12" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="483" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B483" s="8"/>
-    </row>
-    <row r="484" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B484" s="8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="485" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B485" s="8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="486" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B486" s="8" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="487" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="488" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="489" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="490" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="491" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="492" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="493" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="494" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="495" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="496" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="481" ht="14.25" customHeight="1"/>
+    <row r="482" ht="14.25" customHeight="1"/>
+    <row r="483" ht="14.25" customHeight="1"/>
+    <row r="484" ht="14.25" customHeight="1"/>
+    <row r="485" ht="14.25" customHeight="1"/>
+    <row r="486" ht="14.25" customHeight="1"/>
+    <row r="487" ht="14.25" customHeight="1"/>
+    <row r="488" ht="14.25" customHeight="1"/>
+    <row r="489" ht="14.25" customHeight="1"/>
+    <row r="490" ht="14.25" customHeight="1"/>
+    <row r="491" ht="14.25" customHeight="1"/>
+    <row r="492" ht="14.25" customHeight="1"/>
+    <row r="493" ht="14.25" customHeight="1"/>
+    <row r="494" ht="14.25" customHeight="1"/>
+    <row r="495" ht="14.25" customHeight="1"/>
+    <row r="496" ht="14.25" customHeight="1"/>
     <row r="497" ht="14.25" customHeight="1"/>
     <row r="498" ht="14.25" customHeight="1"/>
     <row r="499" ht="14.25" customHeight="1"/>
@@ -7095,53 +7259,221 @@
     <row r="1038" ht="14.25" customHeight="1"/>
     <row r="1039" ht="14.25" customHeight="1"/>
     <row r="1040" ht="14.25" customHeight="1"/>
-    <row r="1041" ht="14.25" customHeight="1"/>
-    <row r="1042" ht="14.25" customHeight="1"/>
-    <row r="1043" ht="14.25" customHeight="1"/>
-    <row r="1044" ht="14.25" customHeight="1"/>
-    <row r="1045" ht="14.25" customHeight="1"/>
-    <row r="1046" ht="14.25" customHeight="1"/>
-    <row r="1047" ht="14.25" customHeight="1"/>
-    <row r="1048" ht="14.25" customHeight="1"/>
-    <row r="1049" ht="14.25" customHeight="1"/>
-    <row r="1050" ht="14.25" customHeight="1"/>
-    <row r="1051" ht="14.25" customHeight="1"/>
-    <row r="1052" ht="14.25" customHeight="1"/>
-    <row r="1053" ht="14.25" customHeight="1"/>
-    <row r="1054" ht="14.25" customHeight="1"/>
-    <row r="1055" ht="14.25" customHeight="1"/>
-    <row r="1056" ht="14.25" customHeight="1"/>
-    <row r="1057" ht="14.25" customHeight="1"/>
-    <row r="1058" ht="14.25" customHeight="1"/>
-    <row r="1059" ht="14.25" customHeight="1"/>
-    <row r="1060" ht="14.25" customHeight="1"/>
-    <row r="1061" ht="14.25" customHeight="1"/>
-    <row r="1062" ht="14.25" customHeight="1"/>
-    <row r="1063" ht="14.25" customHeight="1"/>
-    <row r="1064" ht="14.25" customHeight="1"/>
-    <row r="1065" ht="14.25" customHeight="1"/>
-    <row r="1066" ht="14.25" customHeight="1"/>
-    <row r="1067" ht="14.25" customHeight="1"/>
-    <row r="1068" ht="14.25" customHeight="1"/>
-    <row r="1069" ht="14.25" customHeight="1"/>
-    <row r="1070" ht="14.25" customHeight="1"/>
-    <row r="1071" ht="14.25" customHeight="1"/>
-    <row r="1072" ht="14.25" customHeight="1"/>
-    <row r="1073" ht="14.25" customHeight="1"/>
-    <row r="1074" ht="14.25" customHeight="1"/>
-    <row r="1075" ht="14.25" customHeight="1"/>
-    <row r="1076" ht="14.25" customHeight="1"/>
-    <row r="1077" ht="14.25" customHeight="1"/>
-    <row r="1078" ht="14.25" customHeight="1"/>
-    <row r="1079" ht="14.25" customHeight="1"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B19" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A4:C7"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="2" max="2" width="32.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C4" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>189</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B3:B41"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="3" spans="2:2">
+      <c r="B3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2">
+      <c r="B4" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2">
+      <c r="B5" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2">
+      <c r="B7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2">
+      <c r="B8" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2">
+      <c r="B9" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2">
+      <c r="B11" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2">
+      <c r="B12" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2">
+      <c r="B13" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2">
+      <c r="B15" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2">
+      <c r="B16" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2">
+      <c r="B19" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2">
+      <c r="B21" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2">
+      <c r="B23" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2">
+      <c r="B24" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2">
+      <c r="B25" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2">
+      <c r="B27" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="28" spans="2:2">
+      <c r="B28" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2">
+      <c r="B29" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2">
+      <c r="B31" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2">
+      <c r="B37" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2">
+      <c r="B38" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2">
+      <c r="B40" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2">
+      <c r="B41" t="s">
+        <v>217</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="C65:Q116"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -7153,12 +7485,12 @@
   </cols>
   <sheetData>
     <row r="65" spans="3:17">
-      <c r="N65" s="27" t="s">
+      <c r="N65" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="O65" s="27"/>
-      <c r="P65" s="27"/>
-      <c r="Q65" s="27"/>
+      <c r="O65" s="25"/>
+      <c r="P65" s="25"/>
+      <c r="Q65" s="25"/>
     </row>
     <row r="69" spans="3:17">
       <c r="C69" s="26" t="s">
@@ -7181,12 +7513,12 @@
       <c r="D70" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="E70" s="28" t="s">
+      <c r="E70" s="27" t="s">
         <v>89</v>
       </c>
-      <c r="F70" s="28"/>
-      <c r="G70" s="28"/>
-      <c r="H70" s="28"/>
+      <c r="F70" s="27"/>
+      <c r="G70" s="27"/>
+      <c r="H70" s="27"/>
       <c r="I70" s="17"/>
       <c r="J70" s="17"/>
       <c r="K70" s="17"/>
@@ -7308,7 +7640,7 @@
         <v>76</v>
       </c>
       <c r="E77" s="24" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F77" s="24"/>
       <c r="G77" s="24"/>
@@ -7401,19 +7733,19 @@
     </row>
     <row r="84" spans="3:13">
       <c r="C84" s="22" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D84" s="23" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="E84" s="26" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F84" s="26"/>
       <c r="G84" s="26"/>
       <c r="H84" s="26"/>
       <c r="I84" s="26" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="J84" s="26"/>
       <c r="K84" s="26"/>
@@ -7423,16 +7755,16 @@
         <v>1</v>
       </c>
       <c r="D85" s="19" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E85" s="24" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F85" s="24"/>
       <c r="G85" s="24"/>
       <c r="H85" s="24"/>
       <c r="I85" s="24" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="J85" s="24"/>
       <c r="K85" s="24"/>
@@ -7442,16 +7774,16 @@
         <v>2</v>
       </c>
       <c r="D86" s="19" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E86" s="24" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F86" s="24"/>
       <c r="G86" s="24"/>
       <c r="H86" s="24"/>
       <c r="I86" s="24" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="J86" s="24"/>
       <c r="K86" s="24"/>
@@ -7461,16 +7793,16 @@
         <v>3</v>
       </c>
       <c r="D87" s="19" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E87" s="24" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F87" s="24"/>
       <c r="G87" s="24"/>
       <c r="H87" s="24"/>
       <c r="I87" s="24" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="J87" s="24"/>
       <c r="K87" s="24"/>
@@ -7480,16 +7812,16 @@
         <v>4</v>
       </c>
       <c r="D88" s="19" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E88" s="24" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F88" s="24"/>
       <c r="G88" s="24"/>
       <c r="H88" s="24"/>
       <c r="I88" s="24" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="J88" s="24"/>
       <c r="K88" s="24"/>
@@ -7499,16 +7831,16 @@
         <v>5</v>
       </c>
       <c r="D89" s="19" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="E89" s="24" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F89" s="24"/>
       <c r="G89" s="24"/>
       <c r="H89" s="24"/>
       <c r="I89" s="24" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="J89" s="24"/>
       <c r="K89" s="24"/>
@@ -7518,16 +7850,16 @@
         <v>6</v>
       </c>
       <c r="D90" s="19" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E90" s="24" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F90" s="24"/>
       <c r="G90" s="24"/>
       <c r="H90" s="24"/>
       <c r="I90" s="24" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="J90" s="24"/>
       <c r="K90" s="24"/>
@@ -7537,16 +7869,16 @@
         <v>7</v>
       </c>
       <c r="D91" s="19" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E91" s="24" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="F91" s="24"/>
       <c r="G91" s="24"/>
       <c r="H91" s="24"/>
       <c r="I91" s="24" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="J91" s="24"/>
       <c r="K91" s="24"/>
@@ -7556,16 +7888,16 @@
         <v>8</v>
       </c>
       <c r="D92" s="19" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E92" s="24" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F92" s="24"/>
       <c r="G92" s="24"/>
       <c r="H92" s="24"/>
       <c r="I92" s="24" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="J92" s="24"/>
       <c r="K92" s="24"/>
@@ -7575,16 +7907,16 @@
         <v>9</v>
       </c>
       <c r="D93" s="19" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="E93" s="24" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="F93" s="24"/>
       <c r="G93" s="24"/>
       <c r="H93" s="24"/>
       <c r="I93" s="24" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="J93" s="24"/>
       <c r="K93" s="24"/>
@@ -7594,16 +7926,16 @@
         <v>10</v>
       </c>
       <c r="D94" s="19" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E94" s="24" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="F94" s="24"/>
       <c r="G94" s="24"/>
       <c r="H94" s="24"/>
       <c r="I94" s="24" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J94" s="24"/>
       <c r="K94" s="24"/>
@@ -7613,16 +7945,16 @@
         <v>11</v>
       </c>
       <c r="D95" s="19" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E95" s="24" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F95" s="24"/>
       <c r="G95" s="24"/>
       <c r="H95" s="24"/>
       <c r="I95" s="24" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="J95" s="24"/>
       <c r="K95" s="24"/>
@@ -7632,16 +7964,16 @@
         <v>12</v>
       </c>
       <c r="D96" s="19" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="E96" s="24" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F96" s="24"/>
       <c r="G96" s="24"/>
       <c r="H96" s="24"/>
       <c r="I96" s="24" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="J96" s="24"/>
       <c r="K96" s="24"/>
@@ -7651,16 +7983,16 @@
         <v>13</v>
       </c>
       <c r="D97" s="19" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E97" s="24" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="F97" s="24"/>
       <c r="G97" s="24"/>
       <c r="H97" s="24"/>
       <c r="I97" s="24" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="J97" s="24"/>
       <c r="K97" s="24"/>
@@ -7670,16 +8002,16 @@
         <v>14</v>
       </c>
       <c r="D98" s="19" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E98" s="24" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="F98" s="24"/>
       <c r="G98" s="24"/>
       <c r="H98" s="24"/>
       <c r="I98" s="24" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="J98" s="24"/>
       <c r="K98" s="24"/>
@@ -7689,16 +8021,16 @@
         <v>15</v>
       </c>
       <c r="D99" s="19" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="E99" s="24" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F99" s="24"/>
       <c r="G99" s="24"/>
       <c r="H99" s="24"/>
       <c r="I99" s="24" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="J99" s="24"/>
       <c r="K99" s="24"/>
@@ -7708,16 +8040,16 @@
         <v>16</v>
       </c>
       <c r="D100" s="19" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E100" s="24" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="F100" s="24"/>
       <c r="G100" s="24"/>
       <c r="H100" s="24"/>
       <c r="I100" s="24" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="J100" s="24"/>
       <c r="K100" s="24"/>
@@ -7727,16 +8059,16 @@
         <v>17</v>
       </c>
       <c r="D101" s="19" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E101" s="24" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="F101" s="24"/>
       <c r="G101" s="24"/>
       <c r="H101" s="24"/>
       <c r="I101" s="24" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="J101" s="24"/>
       <c r="K101" s="24"/>
@@ -7746,16 +8078,16 @@
         <v>18</v>
       </c>
       <c r="D102" s="19" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="E102" s="24" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="F102" s="24"/>
       <c r="G102" s="24"/>
       <c r="H102" s="24"/>
       <c r="I102" s="24" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J102" s="24"/>
       <c r="K102" s="24"/>
@@ -7765,16 +8097,16 @@
         <v>19</v>
       </c>
       <c r="D103" s="19" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E103" s="24" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="F103" s="24"/>
       <c r="G103" s="24"/>
       <c r="H103" s="24"/>
       <c r="I103" s="24" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="J103" s="24"/>
       <c r="K103" s="24"/>
@@ -7784,16 +8116,16 @@
         <v>20</v>
       </c>
       <c r="D104" s="19" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="E104" s="24" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="F104" s="24"/>
       <c r="G104" s="24"/>
       <c r="H104" s="24"/>
       <c r="I104" s="24" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="J104" s="24"/>
       <c r="K104" s="24"/>
@@ -7803,16 +8135,16 @@
         <v>21</v>
       </c>
       <c r="D105" s="19" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E105" s="24" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="F105" s="24"/>
       <c r="G105" s="24"/>
       <c r="H105" s="24"/>
       <c r="I105" s="24" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="J105" s="24"/>
       <c r="K105" s="24"/>
@@ -7822,16 +8154,16 @@
         <v>22</v>
       </c>
       <c r="D106" s="19" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E106" s="24" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="F106" s="24"/>
       <c r="G106" s="24"/>
       <c r="H106" s="24"/>
       <c r="I106" s="24" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="J106" s="24"/>
       <c r="K106" s="24"/>
@@ -7841,16 +8173,16 @@
         <v>23</v>
       </c>
       <c r="D107" s="19" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E107" s="24" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="F107" s="24"/>
       <c r="G107" s="24"/>
       <c r="H107" s="24"/>
       <c r="I107" s="24" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="J107" s="24"/>
       <c r="K107" s="24"/>
@@ -7860,16 +8192,16 @@
         <v>24</v>
       </c>
       <c r="D108" s="19" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E108" s="24" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="F108" s="24"/>
       <c r="G108" s="24"/>
       <c r="H108" s="24"/>
       <c r="I108" s="24" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="J108" s="24"/>
       <c r="K108" s="24"/>
@@ -7879,16 +8211,16 @@
         <v>25</v>
       </c>
       <c r="D109" s="19" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="E109" s="24" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F109" s="24"/>
       <c r="G109" s="24"/>
       <c r="H109" s="24"/>
       <c r="I109" s="24" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J109" s="24"/>
       <c r="K109" s="24"/>
@@ -7898,16 +8230,16 @@
         <v>26</v>
       </c>
       <c r="D110" s="19" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E110" s="24" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F110" s="24"/>
       <c r="G110" s="24"/>
       <c r="H110" s="24"/>
       <c r="I110" s="24" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="J110" s="24"/>
       <c r="K110" s="24"/>
@@ -7917,16 +8249,16 @@
         <v>27</v>
       </c>
       <c r="D111" s="19" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E111" s="24" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="F111" s="24"/>
       <c r="G111" s="24"/>
       <c r="H111" s="24"/>
       <c r="I111" s="24" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="J111" s="24"/>
       <c r="K111" s="24"/>
@@ -7936,16 +8268,16 @@
         <v>28</v>
       </c>
       <c r="D112" s="19" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="E112" s="24" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="F112" s="24"/>
       <c r="G112" s="24"/>
       <c r="H112" s="24"/>
       <c r="I112" s="24" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="J112" s="24"/>
       <c r="K112" s="24"/>
@@ -7955,40 +8287,105 @@
         <v>29</v>
       </c>
       <c r="D113" s="19" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="E113" s="24" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="F113" s="24"/>
       <c r="G113" s="24"/>
       <c r="H113" s="24"/>
       <c r="I113" s="24" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="J113" s="24"/>
       <c r="K113" s="24"/>
     </row>
     <row r="114" spans="3:11">
-      <c r="E114" s="25"/>
-      <c r="F114" s="25"/>
-      <c r="G114" s="25"/>
-      <c r="H114" s="25"/>
+      <c r="E114" s="28"/>
+      <c r="F114" s="28"/>
+      <c r="G114" s="28"/>
+      <c r="H114" s="28"/>
     </row>
     <row r="115" spans="3:11">
-      <c r="E115" s="25"/>
-      <c r="F115" s="25"/>
-      <c r="G115" s="25"/>
-      <c r="H115" s="25"/>
+      <c r="E115" s="28"/>
+      <c r="F115" s="28"/>
+      <c r="G115" s="28"/>
+      <c r="H115" s="28"/>
     </row>
     <row r="116" spans="3:11">
-      <c r="E116" s="25"/>
-      <c r="F116" s="25"/>
-      <c r="G116" s="25"/>
-      <c r="H116" s="25"/>
+      <c r="E116" s="28"/>
+      <c r="F116" s="28"/>
+      <c r="G116" s="28"/>
+      <c r="H116" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="77">
+    <mergeCell ref="E113:H113"/>
+    <mergeCell ref="I113:K113"/>
+    <mergeCell ref="E114:H114"/>
+    <mergeCell ref="E115:H115"/>
+    <mergeCell ref="E116:H116"/>
+    <mergeCell ref="E110:H110"/>
+    <mergeCell ref="I110:K110"/>
+    <mergeCell ref="E111:H111"/>
+    <mergeCell ref="I111:K111"/>
+    <mergeCell ref="E112:H112"/>
+    <mergeCell ref="I112:K112"/>
+    <mergeCell ref="E107:H107"/>
+    <mergeCell ref="I107:K107"/>
+    <mergeCell ref="E108:H108"/>
+    <mergeCell ref="I108:K108"/>
+    <mergeCell ref="E109:H109"/>
+    <mergeCell ref="I109:K109"/>
+    <mergeCell ref="E104:H104"/>
+    <mergeCell ref="I104:K104"/>
+    <mergeCell ref="E105:H105"/>
+    <mergeCell ref="I105:K105"/>
+    <mergeCell ref="E106:H106"/>
+    <mergeCell ref="I106:K106"/>
+    <mergeCell ref="E101:H101"/>
+    <mergeCell ref="I101:K101"/>
+    <mergeCell ref="E102:H102"/>
+    <mergeCell ref="I102:K102"/>
+    <mergeCell ref="E103:H103"/>
+    <mergeCell ref="I103:K103"/>
+    <mergeCell ref="E98:H98"/>
+    <mergeCell ref="I98:K98"/>
+    <mergeCell ref="E99:H99"/>
+    <mergeCell ref="I99:K99"/>
+    <mergeCell ref="E100:H100"/>
+    <mergeCell ref="I100:K100"/>
+    <mergeCell ref="E95:H95"/>
+    <mergeCell ref="I95:K95"/>
+    <mergeCell ref="E96:H96"/>
+    <mergeCell ref="I96:K96"/>
+    <mergeCell ref="E97:H97"/>
+    <mergeCell ref="I97:K97"/>
+    <mergeCell ref="E92:H92"/>
+    <mergeCell ref="I92:K92"/>
+    <mergeCell ref="E93:H93"/>
+    <mergeCell ref="I93:K93"/>
+    <mergeCell ref="E94:H94"/>
+    <mergeCell ref="I94:K94"/>
+    <mergeCell ref="E89:H89"/>
+    <mergeCell ref="I89:K89"/>
+    <mergeCell ref="E90:H90"/>
+    <mergeCell ref="I90:K90"/>
+    <mergeCell ref="E91:H91"/>
+    <mergeCell ref="I91:K91"/>
+    <mergeCell ref="E86:H86"/>
+    <mergeCell ref="I86:K86"/>
+    <mergeCell ref="E87:H87"/>
+    <mergeCell ref="I87:K87"/>
+    <mergeCell ref="E88:H88"/>
+    <mergeCell ref="I88:K88"/>
+    <mergeCell ref="E80:H80"/>
+    <mergeCell ref="E81:H81"/>
+    <mergeCell ref="E84:H84"/>
+    <mergeCell ref="I84:K84"/>
+    <mergeCell ref="E85:H85"/>
+    <mergeCell ref="I85:K85"/>
     <mergeCell ref="E79:H79"/>
     <mergeCell ref="N65:Q65"/>
     <mergeCell ref="C69:H69"/>
@@ -8001,71 +8398,6 @@
     <mergeCell ref="E76:H76"/>
     <mergeCell ref="E77:H77"/>
     <mergeCell ref="E78:H78"/>
-    <mergeCell ref="E80:H80"/>
-    <mergeCell ref="E81:H81"/>
-    <mergeCell ref="E84:H84"/>
-    <mergeCell ref="I84:K84"/>
-    <mergeCell ref="E85:H85"/>
-    <mergeCell ref="I85:K85"/>
-    <mergeCell ref="E86:H86"/>
-    <mergeCell ref="I86:K86"/>
-    <mergeCell ref="E87:H87"/>
-    <mergeCell ref="I87:K87"/>
-    <mergeCell ref="E88:H88"/>
-    <mergeCell ref="I88:K88"/>
-    <mergeCell ref="E89:H89"/>
-    <mergeCell ref="I89:K89"/>
-    <mergeCell ref="E90:H90"/>
-    <mergeCell ref="I90:K90"/>
-    <mergeCell ref="E91:H91"/>
-    <mergeCell ref="I91:K91"/>
-    <mergeCell ref="E92:H92"/>
-    <mergeCell ref="I92:K92"/>
-    <mergeCell ref="E93:H93"/>
-    <mergeCell ref="I93:K93"/>
-    <mergeCell ref="E94:H94"/>
-    <mergeCell ref="I94:K94"/>
-    <mergeCell ref="E95:H95"/>
-    <mergeCell ref="I95:K95"/>
-    <mergeCell ref="E96:H96"/>
-    <mergeCell ref="I96:K96"/>
-    <mergeCell ref="E97:H97"/>
-    <mergeCell ref="I97:K97"/>
-    <mergeCell ref="E98:H98"/>
-    <mergeCell ref="I98:K98"/>
-    <mergeCell ref="E99:H99"/>
-    <mergeCell ref="I99:K99"/>
-    <mergeCell ref="E100:H100"/>
-    <mergeCell ref="I100:K100"/>
-    <mergeCell ref="E101:H101"/>
-    <mergeCell ref="I101:K101"/>
-    <mergeCell ref="E102:H102"/>
-    <mergeCell ref="I102:K102"/>
-    <mergeCell ref="E103:H103"/>
-    <mergeCell ref="I103:K103"/>
-    <mergeCell ref="E104:H104"/>
-    <mergeCell ref="I104:K104"/>
-    <mergeCell ref="E105:H105"/>
-    <mergeCell ref="I105:K105"/>
-    <mergeCell ref="E106:H106"/>
-    <mergeCell ref="I106:K106"/>
-    <mergeCell ref="E107:H107"/>
-    <mergeCell ref="I107:K107"/>
-    <mergeCell ref="E108:H108"/>
-    <mergeCell ref="I108:K108"/>
-    <mergeCell ref="E109:H109"/>
-    <mergeCell ref="I109:K109"/>
-    <mergeCell ref="E110:H110"/>
-    <mergeCell ref="I110:K110"/>
-    <mergeCell ref="E111:H111"/>
-    <mergeCell ref="I111:K111"/>
-    <mergeCell ref="E112:H112"/>
-    <mergeCell ref="I112:K112"/>
-    <mergeCell ref="E113:H113"/>
-    <mergeCell ref="I113:K113"/>
-    <mergeCell ref="E114:H114"/>
-    <mergeCell ref="E115:H115"/>
-    <mergeCell ref="E116:H116"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>